<commit_message>
Update backwrite template.xlsx with user edits
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/backwrite/template.xlsx
+++ b/src/backwrite/template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work Temp\!New\!backwrite test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\scrib\dev\ctv-orderentry\src\backwrite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75C339B5-2CF2-4386-A4AD-E3D66DD06FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5488E2A2-4ED9-4949-8121-9E00CEEBEEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="615" windowWidth="21135" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales Confirmation" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -705,7 +705,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -882,15 +882,6 @@
       <bottom style="double">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1132,7 +1123,7 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1178,15 +1169,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1218,10 +1200,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1234,14 +1213,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="70" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1250,7 +1229,7 @@
     <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="55" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1297,9 +1276,33 @@
     <xf numFmtId="7" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="23" xfId="70" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="22" xfId="70" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1308,53 +1311,51 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="89">
@@ -2397,7 +2398,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:C6" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="29">
     <pivotField showAll="0"/>
@@ -2820,35 +2821,35 @@
   <dimension ref="A1:AJ36"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" style="32" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="11" style="33" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="33" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" style="33" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" style="33" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.28515625" style="32" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="33" customWidth="1"/>
-    <col min="10" max="10" width="5.85546875" style="33" customWidth="1"/>
-    <col min="11" max="11" width="6.42578125" style="33" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="10" style="33" customWidth="1"/>
-    <col min="13" max="13" width="10" style="33" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="11.5703125" style="33" customWidth="1"/>
-    <col min="16" max="16" width="13.5703125" style="33" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" style="33" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.85546875" style="32" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="6.7109375" style="32" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="10.5703125" style="32" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="26.5703125" style="32" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="10.140625" style="32" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="11" style="32" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="11.7109375" style="32" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="10.140625" style="32" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="7.140625" style="32" hidden="1" customWidth="1"/>
-    <col min="27" max="28" width="8.42578125" style="32" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="6.42578125" style="32" hidden="1" customWidth="1"/>
-    <col min="30" max="36" width="0" style="32" hidden="1" customWidth="1"/>
-    <col min="37" max="16384" width="149.140625" style="32" hidden="1"/>
+    <col min="1" max="1" width="23.28515625" style="28" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="11" style="29" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="29" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="29" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" style="29" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.140625" style="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.28515625" style="28" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="29" customWidth="1"/>
+    <col min="10" max="10" width="5.85546875" style="29" customWidth="1"/>
+    <col min="11" max="11" width="6.42578125" style="29" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="10" style="29" customWidth="1"/>
+    <col min="13" max="13" width="10" style="29" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="11.5703125" style="29" customWidth="1"/>
+    <col min="16" max="16" width="14" style="29" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" style="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" style="28" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="6.7109375" style="28" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="10.5703125" style="28" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="26.5703125" style="28" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" style="28" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="11" style="28" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="11.7109375" style="28" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="10.140625" style="28" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="7.140625" style="28" hidden="1" customWidth="1"/>
+    <col min="27" max="28" width="8.42578125" style="28" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="6.42578125" style="28" hidden="1" customWidth="1"/>
+    <col min="30" max="36" width="0" style="28" hidden="1" customWidth="1"/>
+    <col min="37" max="16384" width="149.140625" style="28" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2856,15 +2857,15 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="79" t="s">
+      <c r="F1" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
@@ -2893,48 +2894,48 @@
         <v>0</v>
       </c>
       <c r="C3" s="2"/>
-      <c r="D3" s="80" t="s">
+      <c r="D3" s="63" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
       <c r="I3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
-      <c r="L3" s="81" t="s">
+      <c r="L3" s="64" t="s">
         <v>75</v>
       </c>
-      <c r="M3" s="81"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81"/>
-      <c r="P3" s="81"/>
-      <c r="Q3" s="81"/>
+      <c r="M3" s="64"/>
+      <c r="N3" s="64"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
     </row>
     <row r="4" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="82" t="s">
+      <c r="D4" s="71" t="s">
         <v>112</v>
       </c>
-      <c r="E4" s="82"/>
-      <c r="F4" s="82"/>
-      <c r="G4" s="82"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="71"/>
       <c r="I4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="81" t="s">
+      <c r="L4" s="64" t="s">
         <v>78</v>
       </c>
-      <c r="M4" s="81"/>
-      <c r="N4" s="81"/>
-      <c r="O4" s="81"/>
-      <c r="P4" s="81"/>
-      <c r="Q4" s="81"/>
+      <c r="M4" s="64"/>
+      <c r="N4" s="64"/>
+      <c r="O4" s="64"/>
+      <c r="P4" s="64"/>
+      <c r="Q4" s="64"/>
     </row>
     <row r="5" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
@@ -2952,26 +2953,26 @@
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
-      <c r="L5" s="81" t="s">
+      <c r="L5" s="64" t="s">
         <v>77</v>
       </c>
-      <c r="M5" s="81"/>
-      <c r="N5" s="81"/>
-      <c r="O5" s="81"/>
-      <c r="P5" s="81"/>
-      <c r="Q5" s="81"/>
+      <c r="M5" s="64"/>
+      <c r="N5" s="64"/>
+      <c r="O5" s="64"/>
+      <c r="P5" s="64"/>
+      <c r="Q5" s="64"/>
     </row>
     <row r="6" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="80" t="s">
+      <c r="D6" s="63" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="80"/>
-      <c r="F6" s="51" t="s">
+      <c r="E6" s="63"/>
+      <c r="F6" s="47" t="s">
         <v>73</v>
       </c>
-      <c r="G6" s="51" t="s">
+      <c r="G6" s="47" t="s">
         <v>74</v>
       </c>
       <c r="I6" s="3" t="s">
@@ -2979,14 +2980,14 @@
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
-      <c r="L6" s="81" t="s">
+      <c r="L6" s="64" t="s">
         <v>79</v>
       </c>
-      <c r="M6" s="81"/>
-      <c r="N6" s="81"/>
-      <c r="O6" s="81"/>
-      <c r="P6" s="81"/>
-      <c r="Q6" s="81"/>
+      <c r="M6" s="64"/>
+      <c r="N6" s="64"/>
+      <c r="O6" s="64"/>
+      <c r="P6" s="64"/>
+      <c r="Q6" s="64"/>
     </row>
     <row r="7" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
@@ -3001,37 +3002,37 @@
         <v>6</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="85" t="s">
+      <c r="D8" s="67" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="85"/>
-      <c r="F8" s="85"/>
-      <c r="G8" s="85"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="67"/>
+      <c r="G8" s="67"/>
       <c r="I8" s="3" t="s">
         <v>45</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
-      <c r="L8" s="84" t="s">
+      <c r="L8" s="66" t="s">
         <v>76</v>
       </c>
-      <c r="M8" s="84"/>
-      <c r="N8" s="84"/>
-      <c r="O8" s="84"/>
-      <c r="P8" s="84"/>
-      <c r="Q8" s="84"/>
+      <c r="M8" s="66"/>
+      <c r="N8" s="66"/>
+      <c r="O8" s="66"/>
+      <c r="P8" s="66"/>
+      <c r="Q8" s="66"/>
     </row>
     <row r="9" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="85" t="s">
+      <c r="D9" s="67" t="s">
         <v>107</v>
       </c>
-      <c r="E9" s="85"/>
-      <c r="F9" s="85"/>
-      <c r="G9" s="85"/>
+      <c r="E9" s="67"/>
+      <c r="F9" s="67"/>
+      <c r="G9" s="67"/>
       <c r="I9" s="3" t="s">
         <v>10</v>
       </c>
@@ -3051,12 +3052,12 @@
         <v>9</v>
       </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="67" t="s">
+      <c r="D10" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="68"/>
-      <c r="F10" s="68"/>
-      <c r="G10" s="68"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="69"/>
       <c r="I10" s="3" t="s">
         <v>47</v>
       </c>
@@ -3069,37 +3070,37 @@
         <v>9</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="67" t="s">
+      <c r="D11" s="68" t="s">
         <v>109</v>
       </c>
-      <c r="E11" s="68"/>
-      <c r="F11" s="68"/>
-      <c r="G11" s="68"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
       <c r="I11" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J11" s="2"/>
-      <c r="K11" s="81" t="s">
+      <c r="K11" s="64" t="s">
         <v>69</v>
       </c>
-      <c r="L11" s="81"/>
-      <c r="M11" s="81"/>
-      <c r="N11" s="81"/>
-      <c r="O11" s="81"/>
-      <c r="P11" s="81"/>
-      <c r="Q11" s="81"/>
+      <c r="L11" s="64"/>
+      <c r="M11" s="64"/>
+      <c r="N11" s="64"/>
+      <c r="O11" s="64"/>
+      <c r="P11" s="64"/>
+      <c r="Q11" s="64"/>
     </row>
     <row r="12" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="D12" s="67" t="s">
+      <c r="D12" s="68" t="s">
         <v>110</v>
       </c>
-      <c r="E12" s="68"/>
-      <c r="F12" s="68"/>
-      <c r="G12" s="68"/>
+      <c r="E12" s="69"/>
+      <c r="F12" s="69"/>
+      <c r="G12" s="69"/>
       <c r="I12" s="3"/>
       <c r="J12" s="2"/>
       <c r="K12" s="4"/>
@@ -3115,12 +3116,12 @@
         <v>9</v>
       </c>
       <c r="C13" s="2"/>
-      <c r="D13" s="67" t="s">
+      <c r="D13" s="68" t="s">
         <v>111</v>
       </c>
-      <c r="E13" s="68"/>
-      <c r="F13" s="68"/>
-      <c r="G13" s="68"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="69"/>
       <c r="I13" s="3"/>
       <c r="J13" s="2"/>
       <c r="K13" s="4"/>
@@ -3134,7 +3135,7 @@
     <row r="14" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="38"/>
+      <c r="D14" s="34"/>
       <c r="I14" s="3"/>
       <c r="J14" s="2"/>
       <c r="K14" s="4"/>
@@ -3190,7 +3191,7 @@
       <c r="V15" s="9"/>
     </row>
     <row r="16" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="56">
+      <c r="B16" s="52">
         <v>1</v>
       </c>
       <c r="C16" s="11"/>
@@ -3200,7 +3201,7 @@
       <c r="E16" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="56" t="s">
+      <c r="F16" s="52" t="s">
         <v>82</v>
       </c>
       <c r="G16" s="13" t="s">
@@ -3209,23 +3210,23 @@
       <c r="H16" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="I16" s="56">
+      <c r="I16" s="52">
         <v>1</v>
       </c>
-      <c r="J16" s="56" t="s">
+      <c r="J16" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="L16" s="56" t="e">
+      <c r="L16" s="52" t="e">
         <f t="shared" ref="L16" si="0">F16*I16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N16" s="56" t="s">
+      <c r="N16" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="O16" s="41" t="s">
+      <c r="O16" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="P16" s="41" t="e">
+      <c r="P16" s="37" t="e">
         <f t="shared" ref="P16" si="1">L16*O16</f>
         <v>#VALUE!</v>
       </c>
@@ -3235,7 +3236,7 @@
       <c r="V16" s="14"/>
     </row>
     <row r="17" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="56">
+      <c r="B17" s="52">
         <v>2</v>
       </c>
       <c r="C17" s="11"/>
@@ -3245,7 +3246,7 @@
       <c r="E17" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F17" s="56" t="s">
+      <c r="F17" s="52" t="s">
         <v>82</v>
       </c>
       <c r="G17" s="13" t="s">
@@ -3254,337 +3255,339 @@
       <c r="H17" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="I17" s="56">
+      <c r="I17" s="52">
         <v>1</v>
       </c>
-      <c r="J17" s="56" t="s">
+      <c r="J17" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="L17" s="56" t="e">
+      <c r="L17" s="52" t="e">
         <f t="shared" ref="L17:L19" si="2">F17*I17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N17" s="56" t="s">
+      <c r="N17" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="O17" s="41" t="s">
+      <c r="O17" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="P17" s="41" t="e">
+      <c r="P17" s="37" t="e">
         <f t="shared" ref="P17:P19" si="3">L17*O17</f>
         <v>#VALUE!</v>
       </c>
+      <c r="Q17" s="82"/>
       <c r="R17" s="14"/>
       <c r="T17" s="14"/>
       <c r="U17" s="14"/>
       <c r="V17" s="14"/>
     </row>
     <row r="18" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="56">
+      <c r="B18" s="87">
         <v>3</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12" t="s">
+      <c r="C18" s="88"/>
+      <c r="D18" s="89" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="56" t="s">
+      <c r="F18" s="87" t="s">
         <v>82</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="G18" s="90" t="s">
         <v>114</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="82" t="s">
         <v>113</v>
       </c>
-      <c r="I18" s="56">
+      <c r="I18" s="87">
         <v>1</v>
       </c>
-      <c r="J18" s="56" t="s">
+      <c r="J18" s="87" t="s">
         <v>84</v>
       </c>
-      <c r="L18" s="56" t="e">
+      <c r="L18" s="52" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="N18" s="56" t="s">
+      <c r="N18" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="O18" s="41" t="s">
+      <c r="O18" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="P18" s="41" t="e">
+      <c r="P18" s="37" t="e">
         <f t="shared" si="3"/>
         <v>#VALUE!</v>
       </c>
+      <c r="Q18" s="82"/>
       <c r="R18" s="14"/>
       <c r="T18" s="14"/>
       <c r="U18" s="14"/>
       <c r="V18" s="14"/>
     </row>
     <row r="19" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="56">
+      <c r="B19" s="87">
         <v>4</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12" t="s">
+      <c r="C19" s="88"/>
+      <c r="D19" s="89" t="s">
         <v>80</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="56" t="s">
+      <c r="F19" s="87" t="s">
         <v>82</v>
       </c>
-      <c r="G19" s="13" t="s">
+      <c r="G19" s="90" t="s">
         <v>114</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="82" t="s">
         <v>113</v>
       </c>
-      <c r="I19" s="56">
+      <c r="I19" s="87">
         <v>1</v>
       </c>
-      <c r="J19" s="56" t="s">
+      <c r="J19" s="87" t="s">
         <v>84</v>
       </c>
-      <c r="L19" s="56" t="e">
+      <c r="L19" s="52" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="N19" s="56" t="s">
+      <c r="N19" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="O19" s="41" t="s">
+      <c r="O19" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="P19" s="41" t="e">
+      <c r="P19" s="37" t="e">
         <f t="shared" si="3"/>
         <v>#VALUE!</v>
       </c>
-      <c r="Q19" s="86"/>
+      <c r="Q19" s="82"/>
       <c r="R19" s="14"/>
       <c r="T19" s="14"/>
       <c r="U19" s="14"/>
       <c r="V19" s="14"/>
     </row>
     <row r="20" spans="2:22" s="15" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18" t="s">
+      <c r="B20" s="83"/>
+      <c r="C20" s="83"/>
+      <c r="D20" s="84"/>
+      <c r="E20" s="83"/>
+      <c r="F20" s="83"/>
+      <c r="G20" s="83"/>
+      <c r="H20" s="85"/>
+      <c r="I20" s="85" t="s">
         <v>49</v>
       </c>
-      <c r="J20" s="19"/>
-      <c r="K20" s="35"/>
-      <c r="L20" s="42" t="e">
+      <c r="J20" s="86"/>
+      <c r="K20" s="31"/>
+      <c r="L20" s="38" t="e">
         <f>SUM(L16:L19)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19" t="s">
+      <c r="M20" s="16"/>
+      <c r="N20" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="O20" s="19"/>
-      <c r="P20" s="20" t="s">
+      <c r="O20" s="16"/>
+      <c r="P20" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="Q20" s="87"/>
-    </row>
-    <row r="21" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="83" t="s">
+      <c r="Q20" s="83"/>
+    </row>
+    <row r="21" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="83"/>
-      <c r="D21" s="83"/>
-      <c r="E21" s="83"/>
-      <c r="F21" s="83"/>
-      <c r="G21" s="83"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="23" t="s">
+      <c r="C21" s="65"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="65"/>
+      <c r="G21" s="65"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="J21" s="24"/>
-      <c r="K21" s="36"/>
-      <c r="L21" s="39">
+      <c r="J21" s="21"/>
+      <c r="K21" s="32"/>
+      <c r="L21" s="35">
         <v>0.15</v>
       </c>
-      <c r="M21" s="25"/>
-      <c r="N21" s="25"/>
-      <c r="O21" s="26"/>
-      <c r="P21" s="27" t="e">
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="23"/>
+      <c r="P21" s="24" t="e">
         <f>-1*(L21*P20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Q21" s="28"/>
-    </row>
-    <row r="22" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="69" t="s">
+      <c r="Q21" s="83"/>
+    </row>
+    <row r="22" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="C22" s="70"/>
-      <c r="D22" s="70"/>
-      <c r="E22" s="70"/>
-      <c r="F22" s="70"/>
-      <c r="G22" s="71"/>
+      <c r="C22" s="73"/>
+      <c r="D22" s="73"/>
+      <c r="E22" s="73"/>
+      <c r="F22" s="73"/>
+      <c r="G22" s="74"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="J22" s="22"/>
-      <c r="K22" s="37"/>
-      <c r="L22" s="29"/>
-      <c r="M22" s="30"/>
-      <c r="N22" s="30"/>
-      <c r="O22" s="30"/>
-      <c r="P22" s="31" t="s">
+      <c r="J22" s="19"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="25"/>
+      <c r="M22" s="26"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="26"/>
+      <c r="P22" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="Q22" s="22"/>
-    </row>
-    <row r="23" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="72"/>
-      <c r="C23" s="73"/>
-      <c r="D23" s="73"/>
-      <c r="E23" s="73"/>
-      <c r="F23" s="73"/>
-      <c r="G23" s="74"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="22"/>
-      <c r="N23" s="22"/>
-      <c r="O23" s="22"/>
-      <c r="P23" s="22"/>
-      <c r="Q23" s="22"/>
-    </row>
-    <row r="24" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="72"/>
-      <c r="C24" s="73"/>
-      <c r="D24" s="73"/>
-      <c r="E24" s="73"/>
-      <c r="F24" s="73"/>
-      <c r="G24" s="74"/>
+      <c r="Q22" s="83"/>
+    </row>
+    <row r="23" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="75"/>
+      <c r="C23" s="76"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="76"/>
+      <c r="F23" s="76"/>
+      <c r="G23" s="77"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="19"/>
+      <c r="O23" s="19"/>
+      <c r="P23" s="19"/>
+      <c r="Q23" s="83"/>
+    </row>
+    <row r="24" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="75"/>
+      <c r="C24" s="76"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="77"/>
       <c r="I24" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J24" s="22"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="40"/>
-      <c r="M24" s="40"/>
-      <c r="N24" s="40"/>
-      <c r="O24" s="40"/>
-      <c r="P24" s="40"/>
-      <c r="Q24" s="22"/>
-    </row>
-    <row r="25" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="72"/>
-      <c r="C25" s="73"/>
-      <c r="D25" s="73"/>
-      <c r="E25" s="73"/>
-      <c r="F25" s="73"/>
-      <c r="G25" s="74"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="36"/>
+      <c r="M24" s="36"/>
+      <c r="N24" s="36"/>
+      <c r="O24" s="36"/>
+      <c r="P24" s="36"/>
+      <c r="Q24" s="83"/>
+    </row>
+    <row r="25" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="75"/>
+      <c r="C25" s="76"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="77"/>
       <c r="I25" s="3"/>
-      <c r="J25" s="22"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="22"/>
-      <c r="N25" s="22"/>
-      <c r="O25" s="22"/>
-      <c r="P25" s="22"/>
-      <c r="Q25" s="22"/>
-    </row>
-    <row r="26" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="72"/>
-      <c r="C26" s="73"/>
-      <c r="D26" s="73"/>
-      <c r="E26" s="73"/>
-      <c r="F26" s="73"/>
-      <c r="G26" s="74"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="19"/>
+      <c r="N25" s="19"/>
+      <c r="O25" s="19"/>
+      <c r="P25" s="19"/>
+      <c r="Q25" s="83"/>
+    </row>
+    <row r="26" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="75"/>
+      <c r="C26" s="76"/>
+      <c r="D26" s="76"/>
+      <c r="E26" s="76"/>
+      <c r="F26" s="76"/>
+      <c r="G26" s="77"/>
       <c r="I26" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="J26" s="22"/>
-      <c r="K26" s="22"/>
-      <c r="L26" s="40"/>
-      <c r="M26" s="40"/>
-      <c r="N26" s="40"/>
-      <c r="O26" s="40"/>
-      <c r="P26" s="40"/>
-      <c r="Q26" s="22"/>
-    </row>
-    <row r="27" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="75"/>
-      <c r="C27" s="76"/>
-      <c r="D27" s="76"/>
-      <c r="E27" s="76"/>
-      <c r="F27" s="76"/>
-      <c r="G27" s="77"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="34"/>
-      <c r="K27" s="34"/>
-      <c r="L27" s="34"/>
-      <c r="M27" s="34"/>
-      <c r="N27" s="34"/>
-      <c r="O27" s="34"/>
-      <c r="P27" s="34"/>
-      <c r="Q27" s="22"/>
-    </row>
-    <row r="28" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I28" s="34"/>
-      <c r="J28" s="34"/>
-      <c r="K28" s="34"/>
-      <c r="L28" s="34"/>
-      <c r="M28" s="34"/>
-      <c r="N28" s="34"/>
-      <c r="O28" s="34"/>
-      <c r="P28" s="34"/>
-      <c r="Q28" s="22"/>
-    </row>
-    <row r="29" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="78" t="s">
+      <c r="J26" s="19"/>
+      <c r="K26" s="19"/>
+      <c r="L26" s="36"/>
+      <c r="M26" s="36"/>
+      <c r="N26" s="36"/>
+      <c r="O26" s="36"/>
+      <c r="P26" s="36"/>
+      <c r="Q26" s="83"/>
+    </row>
+    <row r="27" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="78"/>
+      <c r="C27" s="79"/>
+      <c r="D27" s="79"/>
+      <c r="E27" s="79"/>
+      <c r="F27" s="79"/>
+      <c r="G27" s="80"/>
+      <c r="I27" s="30"/>
+      <c r="J27" s="30"/>
+      <c r="K27" s="30"/>
+      <c r="L27" s="30"/>
+      <c r="M27" s="30"/>
+      <c r="N27" s="30"/>
+      <c r="O27" s="30"/>
+      <c r="P27" s="30"/>
+      <c r="Q27" s="83"/>
+    </row>
+    <row r="28" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I28" s="30"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
+      <c r="O28" s="30"/>
+      <c r="P28" s="30"/>
+      <c r="Q28" s="83"/>
+    </row>
+    <row r="29" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="81" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="78"/>
-      <c r="D29" s="78"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="34"/>
-      <c r="K29" s="34"/>
-      <c r="L29" s="34"/>
-      <c r="M29" s="34"/>
-      <c r="N29" s="34"/>
-      <c r="O29" s="34"/>
-      <c r="P29" s="34"/>
-      <c r="Q29" s="22"/>
-    </row>
-    <row r="30" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C29" s="81"/>
+      <c r="D29" s="81"/>
+      <c r="E29" s="40"/>
+      <c r="F29" s="40"/>
+      <c r="G29" s="40"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="30"/>
+      <c r="M29" s="30"/>
+      <c r="N29" s="30"/>
+      <c r="O29" s="30"/>
+      <c r="P29" s="30"/>
+      <c r="Q29" s="83"/>
+    </row>
+    <row r="30" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="I30" s="34"/>
-      <c r="J30" s="34"/>
-      <c r="K30" s="34"/>
-      <c r="L30" s="34"/>
-      <c r="M30" s="34"/>
-      <c r="N30" s="34"/>
-      <c r="O30" s="34"/>
-      <c r="P30" s="34"/>
-      <c r="Q30" s="22"/>
-    </row>
-    <row r="31" spans="2:22" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="30"/>
+      <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
+      <c r="M30" s="30"/>
+      <c r="N30" s="30"/>
+      <c r="O30" s="30"/>
+      <c r="P30" s="30"/>
+      <c r="Q30" s="83"/>
+    </row>
+    <row r="31" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>56</v>
       </c>
@@ -3597,113 +3600,113 @@
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="34"/>
-      <c r="K31" s="34"/>
-      <c r="L31" s="34"/>
-      <c r="M31" s="34"/>
-      <c r="N31" s="34"/>
-      <c r="O31" s="34"/>
-      <c r="P31" s="34"/>
-      <c r="Q31" s="22"/>
-    </row>
-    <row r="32" spans="2:22" s="21" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="45" t="s">
+      <c r="I31" s="30"/>
+      <c r="J31" s="30"/>
+      <c r="K31" s="30"/>
+      <c r="L31" s="30"/>
+      <c r="M31" s="30"/>
+      <c r="N31" s="30"/>
+      <c r="O31" s="30"/>
+      <c r="P31" s="30"/>
+      <c r="Q31" s="19"/>
+    </row>
+    <row r="32" spans="2:22" s="18" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="45"/>
-      <c r="D32" s="46">
+      <c r="C32" s="41"/>
+      <c r="D32" s="42">
         <v>700</v>
       </c>
-      <c r="E32" s="48">
+      <c r="E32" s="44">
         <f>D32*0.85</f>
         <v>595</v>
       </c>
-      <c r="I32" s="34"/>
-      <c r="J32" s="34"/>
-      <c r="K32" s="34"/>
-      <c r="L32" s="34"/>
-      <c r="M32" s="34"/>
-      <c r="N32" s="34"/>
-      <c r="O32" s="34"/>
-      <c r="P32" s="34"/>
-      <c r="Q32" s="22"/>
-    </row>
-    <row r="33" spans="2:17" s="21" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="49" t="s">
+      <c r="I32" s="30"/>
+      <c r="J32" s="30"/>
+      <c r="K32" s="30"/>
+      <c r="L32" s="30"/>
+      <c r="M32" s="30"/>
+      <c r="N32" s="30"/>
+      <c r="O32" s="30"/>
+      <c r="P32" s="30"/>
+      <c r="Q32" s="19"/>
+    </row>
+    <row r="33" spans="2:17" s="18" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="47">
+      <c r="C33" s="19"/>
+      <c r="D33" s="43">
         <f>SUM(D32:D32)</f>
         <v>700</v>
       </c>
-      <c r="E33" s="50">
+      <c r="E33" s="46">
         <f>SUM(E32:E32)</f>
         <v>595</v>
       </c>
-      <c r="F33" s="22"/>
-      <c r="G33" s="22"/>
-      <c r="I33" s="22"/>
-      <c r="J33" s="22"/>
-      <c r="K33" s="22"/>
-      <c r="L33" s="22"/>
-      <c r="M33" s="22"/>
-      <c r="N33" s="22"/>
-      <c r="O33" s="22"/>
-      <c r="P33" s="22"/>
-      <c r="Q33" s="22"/>
-    </row>
-    <row r="34" spans="2:17" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="22"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="22"/>
-      <c r="K34" s="22"/>
-      <c r="L34" s="22"/>
-      <c r="M34" s="22"/>
-      <c r="N34" s="22"/>
-      <c r="O34" s="22"/>
-      <c r="P34" s="22"/>
-      <c r="Q34" s="22"/>
-    </row>
-    <row r="35" spans="2:17" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22"/>
-      <c r="I35" s="22"/>
-      <c r="J35" s="22"/>
-      <c r="K35" s="22"/>
-      <c r="L35" s="22"/>
-      <c r="M35" s="22"/>
-      <c r="N35" s="22"/>
-      <c r="O35" s="22"/>
-      <c r="P35" s="22"/>
-      <c r="Q35" s="22"/>
-    </row>
-    <row r="36" spans="2:17" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="22"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="22"/>
-      <c r="K36" s="22"/>
-      <c r="L36" s="22"/>
-      <c r="M36" s="22"/>
-      <c r="N36" s="22"/>
-      <c r="O36" s="22"/>
-      <c r="P36" s="22"/>
-      <c r="Q36" s="22"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="I33" s="19"/>
+      <c r="J33" s="19"/>
+      <c r="K33" s="19"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="19"/>
+      <c r="N33" s="19"/>
+      <c r="O33" s="19"/>
+      <c r="P33" s="19"/>
+      <c r="Q33" s="19"/>
+    </row>
+    <row r="34" spans="2:17" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="19"/>
+      <c r="I34" s="19"/>
+      <c r="J34" s="19"/>
+      <c r="K34" s="19"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="19"/>
+      <c r="N34" s="19"/>
+      <c r="O34" s="19"/>
+      <c r="P34" s="19"/>
+      <c r="Q34" s="19"/>
+    </row>
+    <row r="35" spans="2:17" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="19"/>
+      <c r="I35" s="19"/>
+      <c r="J35" s="19"/>
+      <c r="K35" s="19"/>
+      <c r="L35" s="19"/>
+      <c r="M35" s="19"/>
+      <c r="N35" s="19"/>
+      <c r="O35" s="19"/>
+      <c r="P35" s="19"/>
+      <c r="Q35" s="19"/>
+    </row>
+    <row r="36" spans="2:17" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="19"/>
+      <c r="G36" s="19"/>
+      <c r="I36" s="19"/>
+      <c r="J36" s="19"/>
+      <c r="K36" s="19"/>
+      <c r="L36" s="19"/>
+      <c r="M36" s="19"/>
+      <c r="N36" s="19"/>
+      <c r="O36" s="19"/>
+      <c r="P36" s="19"/>
+      <c r="Q36" s="19"/>
     </row>
   </sheetData>
   <dataConsolidate function="count">
@@ -3712,6 +3715,13 @@
     </dataRefs>
   </dataConsolidate>
   <mergeCells count="19">
+    <mergeCell ref="B22:G27"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="F1:L1"/>
+    <mergeCell ref="D3:G3"/>
+    <mergeCell ref="L3:Q3"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="L4:Q4"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="L5:Q5"/>
     <mergeCell ref="B21:G21"/>
@@ -3721,16 +3731,9 @@
     <mergeCell ref="L6:Q6"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="D10:G10"/>
-    <mergeCell ref="F1:L1"/>
-    <mergeCell ref="D3:G3"/>
-    <mergeCell ref="L3:Q3"/>
-    <mergeCell ref="D4:G4"/>
-    <mergeCell ref="L4:Q4"/>
     <mergeCell ref="D11:G11"/>
     <mergeCell ref="D12:G12"/>
     <mergeCell ref="D13:G13"/>
-    <mergeCell ref="B22:G27"/>
-    <mergeCell ref="B29:D29"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <hyperlinks>
@@ -3766,9 +3769,9 @@
     <col min="16" max="16" width="12.5703125" customWidth="1"/>
     <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="11" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.7109375" style="53" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.7109375" style="49" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="30" style="58" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="30" style="54" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -3834,13 +3837,13 @@
       <c r="R1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="S1" s="52" t="s">
+      <c r="S1" s="48" t="s">
         <v>56</v>
       </c>
       <c r="T1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="U1" s="57" t="s">
+      <c r="U1" s="53" t="s">
         <v>65</v>
       </c>
       <c r="V1" s="9" t="s">
@@ -3861,7 +3864,7 @@
       <c r="AA1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AB1" s="57" t="s">
+      <c r="AB1" s="53" t="s">
         <v>66</v>
       </c>
       <c r="AC1" s="5" t="s">
@@ -3872,29 +3875,29 @@
       <c r="A2" t="s">
         <v>101</v>
       </c>
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="43" t="str">
+      <c r="C2" s="39" t="str">
         <f t="shared" ref="C2" si="0">B2</f>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D2" s="60" t="s">
+      <c r="D2" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="61" t="s">
+      <c r="E2" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F2" s="61" t="s">
+      <c r="F2" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="61" t="s">
+      <c r="G2" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H2" t="s">
         <v>89</v>
       </c>
-      <c r="I2" s="62" t="s">
+      <c r="I2" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J2" t="s">
@@ -3912,22 +3915,22 @@
       <c r="O2" t="s">
         <v>78</v>
       </c>
-      <c r="P2" s="63" t="s">
+      <c r="P2" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R2" s="63" t="s">
+      <c r="R2" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S2" s="64" t="s">
+      <c r="S2" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T2" s="63" t="s">
+      <c r="T2" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U2" s="65" t="s">
+      <c r="U2" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V2" s="63" t="s">
+      <c r="V2" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W2" t="s">
@@ -3945,7 +3948,7 @@
       <c r="AA2" t="s">
         <v>99</v>
       </c>
-      <c r="AB2" s="65" t="s">
+      <c r="AB2" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC2" t="s">
@@ -3956,29 +3959,29 @@
       <c r="A3" t="s">
         <v>101</v>
       </c>
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="43" t="str">
+      <c r="C3" s="39" t="str">
         <f t="shared" ref="C3:C13" si="1">B3</f>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D3" s="60" t="s">
+      <c r="D3" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E3" s="61" t="s">
+      <c r="E3" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F3" s="61" t="s">
+      <c r="F3" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G3" s="61" t="s">
+      <c r="G3" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H3" t="s">
         <v>89</v>
       </c>
-      <c r="I3" s="62" t="s">
+      <c r="I3" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J3" t="s">
@@ -3996,22 +3999,22 @@
       <c r="O3" t="s">
         <v>78</v>
       </c>
-      <c r="P3" s="63" t="s">
+      <c r="P3" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R3" s="63" t="s">
+      <c r="R3" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S3" s="64" t="s">
+      <c r="S3" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T3" s="63" t="s">
+      <c r="T3" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U3" s="65" t="s">
+      <c r="U3" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V3" s="63" t="s">
+      <c r="V3" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W3" t="s">
@@ -4029,7 +4032,7 @@
       <c r="AA3" t="s">
         <v>99</v>
       </c>
-      <c r="AB3" s="65" t="s">
+      <c r="AB3" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC3" t="s">
@@ -4040,29 +4043,29 @@
       <c r="A4" t="s">
         <v>101</v>
       </c>
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C4" s="43" t="str">
+      <c r="C4" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D4" s="60" t="s">
+      <c r="D4" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E4" s="61" t="s">
+      <c r="E4" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F4" s="61" t="s">
+      <c r="F4" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G4" s="61" t="s">
+      <c r="G4" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H4" t="s">
         <v>89</v>
       </c>
-      <c r="I4" s="62" t="s">
+      <c r="I4" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J4" t="s">
@@ -4080,22 +4083,22 @@
       <c r="O4" t="s">
         <v>78</v>
       </c>
-      <c r="P4" s="63" t="s">
+      <c r="P4" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R4" s="63" t="s">
+      <c r="R4" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S4" s="64" t="s">
+      <c r="S4" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T4" s="63" t="s">
+      <c r="T4" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U4" s="65" t="s">
+      <c r="U4" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V4" s="63" t="s">
+      <c r="V4" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W4" t="s">
@@ -4113,7 +4116,7 @@
       <c r="AA4" t="s">
         <v>99</v>
       </c>
-      <c r="AB4" s="65" t="s">
+      <c r="AB4" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC4" t="s">
@@ -4124,29 +4127,29 @@
       <c r="A5" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="59" t="s">
+      <c r="B5" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="43" t="str">
+      <c r="C5" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D5" s="60" t="s">
+      <c r="D5" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E5" s="61" t="s">
+      <c r="E5" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="61" t="s">
+      <c r="F5" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G5" s="61" t="s">
+      <c r="G5" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H5" t="s">
         <v>89</v>
       </c>
-      <c r="I5" s="62" t="s">
+      <c r="I5" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J5" t="s">
@@ -4164,22 +4167,22 @@
       <c r="O5" t="s">
         <v>78</v>
       </c>
-      <c r="P5" s="63" t="s">
+      <c r="P5" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R5" s="63" t="s">
+      <c r="R5" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S5" s="64" t="s">
+      <c r="S5" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T5" s="63" t="s">
+      <c r="T5" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U5" s="65" t="s">
+      <c r="U5" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V5" s="63" t="s">
+      <c r="V5" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W5" t="s">
@@ -4197,7 +4200,7 @@
       <c r="AA5" t="s">
         <v>99</v>
       </c>
-      <c r="AB5" s="65" t="s">
+      <c r="AB5" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC5" t="s">
@@ -4208,29 +4211,29 @@
       <c r="A6" t="s">
         <v>101</v>
       </c>
-      <c r="B6" s="59" t="s">
+      <c r="B6" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="43" t="str">
+      <c r="C6" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D6" s="60" t="s">
+      <c r="D6" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E6" s="61" t="s">
+      <c r="E6" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="61" t="s">
+      <c r="F6" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G6" s="61" t="s">
+      <c r="G6" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H6" t="s">
         <v>89</v>
       </c>
-      <c r="I6" s="62" t="s">
+      <c r="I6" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J6" t="s">
@@ -4248,22 +4251,22 @@
       <c r="O6" t="s">
         <v>78</v>
       </c>
-      <c r="P6" s="63" t="s">
+      <c r="P6" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R6" s="63" t="s">
+      <c r="R6" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S6" s="64" t="s">
+      <c r="S6" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T6" s="63" t="s">
+      <c r="T6" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U6" s="65" t="s">
+      <c r="U6" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V6" s="63" t="s">
+      <c r="V6" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W6" t="s">
@@ -4281,7 +4284,7 @@
       <c r="AA6" t="s">
         <v>99</v>
       </c>
-      <c r="AB6" s="65" t="s">
+      <c r="AB6" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC6" t="s">
@@ -4292,29 +4295,29 @@
       <c r="A7" t="s">
         <v>101</v>
       </c>
-      <c r="B7" s="59" t="s">
+      <c r="B7" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C7" s="43" t="str">
+      <c r="C7" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D7" s="60" t="s">
+      <c r="D7" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G7" s="61" t="s">
+      <c r="G7" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H7" t="s">
         <v>89</v>
       </c>
-      <c r="I7" s="62" t="s">
+      <c r="I7" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J7" t="s">
@@ -4332,22 +4335,22 @@
       <c r="O7" t="s">
         <v>78</v>
       </c>
-      <c r="P7" s="63" t="s">
+      <c r="P7" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R7" s="63" t="s">
+      <c r="R7" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S7" s="64" t="s">
+      <c r="S7" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T7" s="63" t="s">
+      <c r="T7" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U7" s="65" t="s">
+      <c r="U7" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V7" s="63" t="s">
+      <c r="V7" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W7" t="s">
@@ -4365,7 +4368,7 @@
       <c r="AA7" t="s">
         <v>99</v>
       </c>
-      <c r="AB7" s="65" t="s">
+      <c r="AB7" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC7" t="s">
@@ -4376,29 +4379,29 @@
       <c r="A8" t="s">
         <v>101</v>
       </c>
-      <c r="B8" s="59" t="s">
+      <c r="B8" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="43" t="str">
+      <c r="C8" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D8" s="60" t="s">
+      <c r="D8" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E8" s="61" t="s">
+      <c r="E8" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F8" s="61" t="s">
+      <c r="F8" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G8" s="61" t="s">
+      <c r="G8" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H8" t="s">
         <v>89</v>
       </c>
-      <c r="I8" s="62" t="s">
+      <c r="I8" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J8" t="s">
@@ -4416,22 +4419,22 @@
       <c r="O8" t="s">
         <v>78</v>
       </c>
-      <c r="P8" s="63" t="s">
+      <c r="P8" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R8" s="63" t="s">
+      <c r="R8" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S8" s="64" t="s">
+      <c r="S8" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T8" s="63" t="s">
+      <c r="T8" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U8" s="65" t="s">
+      <c r="U8" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V8" s="63" t="s">
+      <c r="V8" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W8" t="s">
@@ -4449,7 +4452,7 @@
       <c r="AA8" t="s">
         <v>99</v>
       </c>
-      <c r="AB8" s="65" t="s">
+      <c r="AB8" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC8" t="s">
@@ -4460,29 +4463,29 @@
       <c r="A9" t="s">
         <v>101</v>
       </c>
-      <c r="B9" s="59" t="s">
+      <c r="B9" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C9" s="43" t="str">
+      <c r="C9" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D9" s="60" t="s">
+      <c r="D9" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E9" s="61" t="s">
+      <c r="E9" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F9" s="61" t="s">
+      <c r="F9" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G9" s="61" t="s">
+      <c r="G9" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H9" t="s">
         <v>89</v>
       </c>
-      <c r="I9" s="62" t="s">
+      <c r="I9" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J9" t="s">
@@ -4500,22 +4503,22 @@
       <c r="O9" t="s">
         <v>78</v>
       </c>
-      <c r="P9" s="63" t="s">
+      <c r="P9" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R9" s="63" t="s">
+      <c r="R9" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S9" s="64" t="s">
+      <c r="S9" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T9" s="63" t="s">
+      <c r="T9" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U9" s="65" t="s">
+      <c r="U9" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V9" s="63" t="s">
+      <c r="V9" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W9" t="s">
@@ -4533,7 +4536,7 @@
       <c r="AA9" t="s">
         <v>99</v>
       </c>
-      <c r="AB9" s="65" t="s">
+      <c r="AB9" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC9" t="s">
@@ -4544,29 +4547,29 @@
       <c r="A10" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="59" t="s">
+      <c r="B10" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="43" t="str">
+      <c r="C10" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D10" s="60" t="s">
+      <c r="D10" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E10" s="61" t="s">
+      <c r="E10" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="61" t="s">
+      <c r="F10" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G10" s="61" t="s">
+      <c r="G10" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H10" t="s">
         <v>89</v>
       </c>
-      <c r="I10" s="62" t="s">
+      <c r="I10" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J10" t="s">
@@ -4584,22 +4587,22 @@
       <c r="O10" t="s">
         <v>78</v>
       </c>
-      <c r="P10" s="63" t="s">
+      <c r="P10" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R10" s="63" t="s">
+      <c r="R10" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S10" s="64" t="s">
+      <c r="S10" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T10" s="63" t="s">
+      <c r="T10" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U10" s="65" t="s">
+      <c r="U10" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V10" s="63" t="s">
+      <c r="V10" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W10" t="s">
@@ -4617,7 +4620,7 @@
       <c r="AA10" t="s">
         <v>99</v>
       </c>
-      <c r="AB10" s="65" t="s">
+      <c r="AB10" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC10" t="s">
@@ -4628,29 +4631,29 @@
       <c r="A11" t="s">
         <v>101</v>
       </c>
-      <c r="B11" s="59" t="s">
+      <c r="B11" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C11" s="43" t="str">
+      <c r="C11" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D11" s="60" t="s">
+      <c r="D11" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E11" s="61" t="s">
+      <c r="E11" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F11" s="61" t="s">
+      <c r="F11" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G11" s="61" t="s">
+      <c r="G11" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H11" t="s">
         <v>89</v>
       </c>
-      <c r="I11" s="62" t="s">
+      <c r="I11" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J11" t="s">
@@ -4668,22 +4671,22 @@
       <c r="O11" t="s">
         <v>78</v>
       </c>
-      <c r="P11" s="63" t="s">
+      <c r="P11" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R11" s="63" t="s">
+      <c r="R11" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S11" s="64" t="s">
+      <c r="S11" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T11" s="63" t="s">
+      <c r="T11" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U11" s="65" t="s">
+      <c r="U11" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V11" s="63" t="s">
+      <c r="V11" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W11" t="s">
@@ -4701,7 +4704,7 @@
       <c r="AA11" t="s">
         <v>99</v>
       </c>
-      <c r="AB11" s="65" t="s">
+      <c r="AB11" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC11" t="s">
@@ -4712,29 +4715,29 @@
       <c r="A12" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="59" t="s">
+      <c r="B12" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C12" s="43" t="str">
+      <c r="C12" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D12" s="60" t="s">
+      <c r="D12" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E12" s="61" t="s">
+      <c r="E12" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F12" s="61" t="s">
+      <c r="F12" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G12" s="61" t="s">
+      <c r="G12" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H12" t="s">
         <v>89</v>
       </c>
-      <c r="I12" s="62" t="s">
+      <c r="I12" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J12" t="s">
@@ -4752,22 +4755,22 @@
       <c r="O12" t="s">
         <v>78</v>
       </c>
-      <c r="P12" s="63" t="s">
+      <c r="P12" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R12" s="63" t="s">
+      <c r="R12" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S12" s="64" t="s">
+      <c r="S12" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T12" s="63" t="s">
+      <c r="T12" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U12" s="65" t="s">
+      <c r="U12" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V12" s="63" t="s">
+      <c r="V12" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W12" t="s">
@@ -4785,7 +4788,7 @@
       <c r="AA12" t="s">
         <v>99</v>
       </c>
-      <c r="AB12" s="65" t="s">
+      <c r="AB12" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC12" t="s">
@@ -4796,29 +4799,29 @@
       <c r="A13" t="s">
         <v>101</v>
       </c>
-      <c r="B13" s="59" t="s">
+      <c r="B13" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="C13" s="43" t="str">
+      <c r="C13" s="39" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D13" s="60" t="s">
+      <c r="D13" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="E13" s="61" t="s">
+      <c r="E13" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="F13" s="61" t="s">
+      <c r="F13" s="57" t="s">
         <v>88</v>
       </c>
-      <c r="G13" s="61" t="s">
+      <c r="G13" s="57" t="s">
         <v>85</v>
       </c>
       <c r="H13" t="s">
         <v>89</v>
       </c>
-      <c r="I13" s="62" t="s">
+      <c r="I13" s="58" t="s">
         <v>90</v>
       </c>
       <c r="J13" t="s">
@@ -4836,22 +4839,22 @@
       <c r="O13" t="s">
         <v>78</v>
       </c>
-      <c r="P13" s="63" t="s">
+      <c r="P13" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="R13" s="63" t="s">
+      <c r="R13" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="S13" s="64" t="s">
+      <c r="S13" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="T13" s="63" t="s">
+      <c r="T13" s="59" t="s">
         <v>94</v>
       </c>
-      <c r="U13" s="65" t="s">
+      <c r="U13" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="V13" s="63" t="s">
+      <c r="V13" s="59" t="s">
         <v>96</v>
       </c>
       <c r="W13" t="s">
@@ -4869,7 +4872,7 @@
       <c r="AA13" t="s">
         <v>99</v>
       </c>
-      <c r="AB13" s="65" t="s">
+      <c r="AB13" s="61" t="s">
         <v>70</v>
       </c>
       <c r="AC13" t="s">
@@ -4877,196 +4880,196 @@
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B14" s="59"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="61"/>
-      <c r="F14" s="61"/>
-      <c r="G14" s="61"/>
-      <c r="I14" s="62"/>
-      <c r="P14" s="66"/>
-      <c r="R14" s="66"/>
-      <c r="S14" s="64"/>
-      <c r="T14" s="66"/>
-      <c r="U14" s="65"/>
-      <c r="V14" s="66"/>
-      <c r="AB14" s="65"/>
+      <c r="B14" s="55"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="I14" s="58"/>
+      <c r="P14" s="62"/>
+      <c r="R14" s="62"/>
+      <c r="S14" s="60"/>
+      <c r="T14" s="62"/>
+      <c r="U14" s="61"/>
+      <c r="V14" s="62"/>
+      <c r="AB14" s="61"/>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B15" s="59"/>
-      <c r="C15" s="43"/>
-      <c r="D15" s="60"/>
-      <c r="E15" s="61"/>
-      <c r="F15" s="61"/>
-      <c r="G15" s="61"/>
-      <c r="I15" s="62"/>
-      <c r="P15" s="66"/>
-      <c r="R15" s="66"/>
-      <c r="S15" s="64"/>
-      <c r="T15" s="66"/>
-      <c r="U15" s="65"/>
-      <c r="V15" s="66"/>
-      <c r="AB15" s="65"/>
+      <c r="B15" s="55"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="57"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
+      <c r="I15" s="58"/>
+      <c r="P15" s="62"/>
+      <c r="R15" s="62"/>
+      <c r="S15" s="60"/>
+      <c r="T15" s="62"/>
+      <c r="U15" s="61"/>
+      <c r="V15" s="62"/>
+      <c r="AB15" s="61"/>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B16" s="59"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="61"/>
-      <c r="F16" s="61"/>
-      <c r="G16" s="61"/>
-      <c r="I16" s="62"/>
-      <c r="P16" s="66"/>
-      <c r="R16" s="66"/>
-      <c r="S16" s="64"/>
-      <c r="T16" s="66"/>
-      <c r="U16" s="65"/>
-      <c r="V16" s="66"/>
-      <c r="AB16" s="65"/>
+      <c r="B16" s="55"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="56"/>
+      <c r="E16" s="57"/>
+      <c r="F16" s="57"/>
+      <c r="G16" s="57"/>
+      <c r="I16" s="58"/>
+      <c r="P16" s="62"/>
+      <c r="R16" s="62"/>
+      <c r="S16" s="60"/>
+      <c r="T16" s="62"/>
+      <c r="U16" s="61"/>
+      <c r="V16" s="62"/>
+      <c r="AB16" s="61"/>
     </row>
     <row r="17" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B17" s="59"/>
-      <c r="C17" s="43"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
-      <c r="I17" s="62"/>
-      <c r="P17" s="66"/>
-      <c r="R17" s="66"/>
-      <c r="S17" s="64"/>
-      <c r="T17" s="66"/>
-      <c r="U17" s="65"/>
-      <c r="V17" s="66"/>
-      <c r="AB17" s="65"/>
+      <c r="B17" s="55"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="56"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="57"/>
+      <c r="G17" s="57"/>
+      <c r="I17" s="58"/>
+      <c r="P17" s="62"/>
+      <c r="R17" s="62"/>
+      <c r="S17" s="60"/>
+      <c r="T17" s="62"/>
+      <c r="U17" s="61"/>
+      <c r="V17" s="62"/>
+      <c r="AB17" s="61"/>
     </row>
     <row r="18" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B18" s="59"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="60"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="61"/>
-      <c r="G18" s="61"/>
-      <c r="I18" s="62"/>
-      <c r="P18" s="66"/>
-      <c r="R18" s="66"/>
-      <c r="S18" s="64"/>
-      <c r="T18" s="66"/>
-      <c r="U18" s="65"/>
-      <c r="V18" s="66"/>
-      <c r="AB18" s="65"/>
+      <c r="B18" s="55"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="57"/>
+      <c r="F18" s="57"/>
+      <c r="G18" s="57"/>
+      <c r="I18" s="58"/>
+      <c r="P18" s="62"/>
+      <c r="R18" s="62"/>
+      <c r="S18" s="60"/>
+      <c r="T18" s="62"/>
+      <c r="U18" s="61"/>
+      <c r="V18" s="62"/>
+      <c r="AB18" s="61"/>
     </row>
     <row r="19" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B19" s="59"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="60"/>
-      <c r="E19" s="61"/>
-      <c r="F19" s="61"/>
-      <c r="G19" s="61"/>
-      <c r="I19" s="62"/>
-      <c r="P19" s="66"/>
-      <c r="R19" s="66"/>
-      <c r="S19" s="64"/>
-      <c r="T19" s="66"/>
-      <c r="U19" s="65"/>
-      <c r="V19" s="66"/>
-      <c r="AB19" s="65"/>
+      <c r="B19" s="55"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="57"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="57"/>
+      <c r="I19" s="58"/>
+      <c r="P19" s="62"/>
+      <c r="R19" s="62"/>
+      <c r="S19" s="60"/>
+      <c r="T19" s="62"/>
+      <c r="U19" s="61"/>
+      <c r="V19" s="62"/>
+      <c r="AB19" s="61"/>
     </row>
     <row r="20" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B20" s="59"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="61"/>
-      <c r="G20" s="61"/>
-      <c r="I20" s="62"/>
-      <c r="P20" s="66"/>
-      <c r="R20" s="66"/>
-      <c r="S20" s="64"/>
-      <c r="T20" s="66"/>
-      <c r="U20" s="65"/>
-      <c r="V20" s="66"/>
-      <c r="AB20" s="65"/>
+      <c r="B20" s="55"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="56"/>
+      <c r="E20" s="57"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="57"/>
+      <c r="I20" s="58"/>
+      <c r="P20" s="62"/>
+      <c r="R20" s="62"/>
+      <c r="S20" s="60"/>
+      <c r="T20" s="62"/>
+      <c r="U20" s="61"/>
+      <c r="V20" s="62"/>
+      <c r="AB20" s="61"/>
     </row>
     <row r="21" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B21" s="59"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="60"/>
-      <c r="E21" s="61"/>
-      <c r="F21" s="61"/>
-      <c r="G21" s="61"/>
-      <c r="I21" s="62"/>
-      <c r="P21" s="66"/>
-      <c r="R21" s="66"/>
-      <c r="S21" s="64"/>
-      <c r="T21" s="66"/>
-      <c r="U21" s="65"/>
-      <c r="V21" s="66"/>
-      <c r="AB21" s="65"/>
+      <c r="B21" s="55"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="56"/>
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="57"/>
+      <c r="I21" s="58"/>
+      <c r="P21" s="62"/>
+      <c r="R21" s="62"/>
+      <c r="S21" s="60"/>
+      <c r="T21" s="62"/>
+      <c r="U21" s="61"/>
+      <c r="V21" s="62"/>
+      <c r="AB21" s="61"/>
     </row>
     <row r="22" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B22" s="59"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="61"/>
-      <c r="F22" s="61"/>
-      <c r="G22" s="61"/>
-      <c r="I22" s="62"/>
-      <c r="P22" s="66"/>
-      <c r="R22" s="66"/>
-      <c r="S22" s="64"/>
-      <c r="T22" s="66"/>
-      <c r="U22" s="65"/>
-      <c r="V22" s="66"/>
-      <c r="AB22" s="65"/>
+      <c r="B22" s="55"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="56"/>
+      <c r="E22" s="57"/>
+      <c r="F22" s="57"/>
+      <c r="G22" s="57"/>
+      <c r="I22" s="58"/>
+      <c r="P22" s="62"/>
+      <c r="R22" s="62"/>
+      <c r="S22" s="60"/>
+      <c r="T22" s="62"/>
+      <c r="U22" s="61"/>
+      <c r="V22" s="62"/>
+      <c r="AB22" s="61"/>
     </row>
     <row r="23" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B23" s="59"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="61"/>
-      <c r="F23" s="61"/>
-      <c r="G23" s="61"/>
-      <c r="I23" s="62"/>
-      <c r="P23" s="66"/>
-      <c r="R23" s="66"/>
-      <c r="S23" s="64"/>
-      <c r="T23" s="66"/>
-      <c r="U23" s="65"/>
-      <c r="V23" s="66"/>
-      <c r="AB23" s="65"/>
+      <c r="B23" s="55"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="57"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="I23" s="58"/>
+      <c r="P23" s="62"/>
+      <c r="R23" s="62"/>
+      <c r="S23" s="60"/>
+      <c r="T23" s="62"/>
+      <c r="U23" s="61"/>
+      <c r="V23" s="62"/>
+      <c r="AB23" s="61"/>
     </row>
     <row r="24" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B24" s="59"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="61"/>
-      <c r="F24" s="61"/>
-      <c r="G24" s="61"/>
-      <c r="I24" s="62"/>
-      <c r="P24" s="66"/>
-      <c r="R24" s="66"/>
-      <c r="S24" s="64"/>
-      <c r="T24" s="66"/>
-      <c r="U24" s="65"/>
-      <c r="V24" s="66"/>
-      <c r="AB24" s="65"/>
+      <c r="B24" s="55"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="56"/>
+      <c r="E24" s="57"/>
+      <c r="F24" s="57"/>
+      <c r="G24" s="57"/>
+      <c r="I24" s="58"/>
+      <c r="P24" s="62"/>
+      <c r="R24" s="62"/>
+      <c r="S24" s="60"/>
+      <c r="T24" s="62"/>
+      <c r="U24" s="61"/>
+      <c r="V24" s="62"/>
+      <c r="AB24" s="61"/>
     </row>
     <row r="25" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B25" s="59"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="61"/>
-      <c r="F25" s="61"/>
-      <c r="G25" s="61"/>
-      <c r="I25" s="62"/>
-      <c r="P25" s="66"/>
-      <c r="R25" s="66"/>
-      <c r="S25" s="64"/>
-      <c r="T25" s="66"/>
-      <c r="U25" s="65"/>
-      <c r="V25" s="66"/>
-      <c r="AB25" s="65"/>
+      <c r="B25" s="55"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="56"/>
+      <c r="E25" s="57"/>
+      <c r="F25" s="57"/>
+      <c r="G25" s="57"/>
+      <c r="I25" s="58"/>
+      <c r="P25" s="62"/>
+      <c r="R25" s="62"/>
+      <c r="S25" s="60"/>
+      <c r="T25" s="62"/>
+      <c r="U25" s="61"/>
+      <c r="V25" s="62"/>
+      <c r="AB25" s="61"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AC1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
@@ -5087,7 +5090,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="50" t="s">
         <v>60</v>
       </c>
       <c r="B3" t="s">
@@ -5101,17 +5104,17 @@
       <c r="A4" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="51"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B5" s="55">
+      <c r="B5" s="51">
         <v>0</v>
       </c>
-      <c r="C5" s="55">
+      <c r="C5" s="51">
         <v>0</v>
       </c>
     </row>
@@ -5119,10 +5122,10 @@
       <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="55">
+      <c r="B6" s="51">
         <v>0</v>
       </c>
-      <c r="C6" s="55">
+      <c r="C6" s="51">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update template.xlsx with user edits
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/backwrite/template.xlsx
+++ b/src/backwrite/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\scrib\dev\ctv-orderentry\src\backwrite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5488E2A2-4ED9-4949-8121-9E00CEEBEEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{976CE6D5-5282-4FCD-A3A0-49780F54A24D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -705,7 +705,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -874,17 +874,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="double">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thick">
         <color indexed="64"/>
       </left>
@@ -922,17 +911,6 @@
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1028,6 +1006,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1123,7 +1110,7 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1179,28 +1166,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1210,26 +1182,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="70" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="55" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1276,14 +1236,44 @@
     <xf numFmtId="7" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1291,71 +1281,50 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="22" xfId="70" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="20" xfId="70" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="89">
@@ -2398,7 +2367,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:C6" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="29">
     <pivotField showAll="0"/>
@@ -2821,35 +2790,35 @@
   <dimension ref="A1:AJ36"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" style="28" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="11" style="29" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="29" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" style="29" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.140625" style="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.28515625" style="28" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="29" customWidth="1"/>
-    <col min="10" max="10" width="5.85546875" style="29" customWidth="1"/>
-    <col min="11" max="11" width="6.42578125" style="29" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="10" style="29" customWidth="1"/>
-    <col min="13" max="13" width="10" style="29" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="11.5703125" style="29" customWidth="1"/>
-    <col min="16" max="16" width="14" style="29" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" style="29" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.85546875" style="28" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="6.7109375" style="28" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="10.5703125" style="28" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="26.5703125" style="28" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="10.140625" style="28" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="11" style="28" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="11.7109375" style="28" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="10.140625" style="28" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="7.140625" style="28" hidden="1" customWidth="1"/>
-    <col min="27" max="28" width="8.42578125" style="28" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="6.42578125" style="28" hidden="1" customWidth="1"/>
-    <col min="30" max="36" width="0" style="28" hidden="1" customWidth="1"/>
-    <col min="37" max="16384" width="149.140625" style="28" hidden="1"/>
+    <col min="1" max="1" width="23.28515625" style="23" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="11" style="24" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="24" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="24" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" style="24" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.28515625" style="23" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="24" customWidth="1"/>
+    <col min="10" max="10" width="5.85546875" style="24" customWidth="1"/>
+    <col min="11" max="11" width="6.42578125" style="24" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="10" style="24" customWidth="1"/>
+    <col min="13" max="13" width="10" style="24" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="11.5703125" style="24" customWidth="1"/>
+    <col min="16" max="16" width="14" style="24" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" style="24" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" style="23" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="6.7109375" style="23" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="10.5703125" style="23" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="26.5703125" style="23" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" style="23" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="11" style="23" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="11.7109375" style="23" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="10.140625" style="23" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="7.140625" style="23" hidden="1" customWidth="1"/>
+    <col min="27" max="28" width="8.42578125" style="23" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="6.42578125" style="23" hidden="1" customWidth="1"/>
+    <col min="30" max="36" width="0" style="23" hidden="1" customWidth="1"/>
+    <col min="37" max="16384" width="149.140625" style="23" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2857,15 +2826,15 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="70" t="s">
+      <c r="F1" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
@@ -2894,48 +2863,48 @@
         <v>0</v>
       </c>
       <c r="C3" s="2"/>
-      <c r="D3" s="63" t="s">
+      <c r="D3" s="64" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
       <c r="I3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
-      <c r="L3" s="64" t="s">
+      <c r="L3" s="65" t="s">
         <v>75</v>
       </c>
-      <c r="M3" s="64"/>
-      <c r="N3" s="64"/>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
+      <c r="M3" s="65"/>
+      <c r="N3" s="65"/>
+      <c r="O3" s="65"/>
+      <c r="P3" s="65"/>
+      <c r="Q3" s="65"/>
     </row>
     <row r="4" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="71" t="s">
+      <c r="D4" s="66" t="s">
         <v>112</v>
       </c>
-      <c r="E4" s="71"/>
-      <c r="F4" s="71"/>
-      <c r="G4" s="71"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
       <c r="I4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="64" t="s">
+      <c r="L4" s="65" t="s">
         <v>78</v>
       </c>
-      <c r="M4" s="64"/>
-      <c r="N4" s="64"/>
-      <c r="O4" s="64"/>
-      <c r="P4" s="64"/>
-      <c r="Q4" s="64"/>
+      <c r="M4" s="65"/>
+      <c r="N4" s="65"/>
+      <c r="O4" s="65"/>
+      <c r="P4" s="65"/>
+      <c r="Q4" s="65"/>
     </row>
     <row r="5" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
@@ -2953,26 +2922,26 @@
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
-      <c r="L5" s="64" t="s">
+      <c r="L5" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="M5" s="64"/>
-      <c r="N5" s="64"/>
-      <c r="O5" s="64"/>
-      <c r="P5" s="64"/>
-      <c r="Q5" s="64"/>
+      <c r="M5" s="65"/>
+      <c r="N5" s="65"/>
+      <c r="O5" s="65"/>
+      <c r="P5" s="65"/>
+      <c r="Q5" s="65"/>
     </row>
     <row r="6" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="63" t="s">
+      <c r="D6" s="64" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="63"/>
-      <c r="F6" s="47" t="s">
+      <c r="E6" s="64"/>
+      <c r="F6" s="38" t="s">
         <v>73</v>
       </c>
-      <c r="G6" s="47" t="s">
+      <c r="G6" s="38" t="s">
         <v>74</v>
       </c>
       <c r="I6" s="3" t="s">
@@ -2980,14 +2949,14 @@
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
-      <c r="L6" s="64" t="s">
+      <c r="L6" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="M6" s="64"/>
-      <c r="N6" s="64"/>
-      <c r="O6" s="64"/>
-      <c r="P6" s="64"/>
-      <c r="Q6" s="64"/>
+      <c r="M6" s="65"/>
+      <c r="N6" s="65"/>
+      <c r="O6" s="65"/>
+      <c r="P6" s="65"/>
+      <c r="Q6" s="65"/>
     </row>
     <row r="7" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
@@ -3002,37 +2971,37 @@
         <v>6</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="67" t="s">
+      <c r="D8" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="67"/>
-      <c r="F8" s="67"/>
-      <c r="G8" s="67"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="68"/>
       <c r="I8" s="3" t="s">
         <v>45</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
-      <c r="L8" s="66" t="s">
+      <c r="L8" s="67" t="s">
         <v>76</v>
       </c>
-      <c r="M8" s="66"/>
-      <c r="N8" s="66"/>
-      <c r="O8" s="66"/>
-      <c r="P8" s="66"/>
-      <c r="Q8" s="66"/>
+      <c r="M8" s="67"/>
+      <c r="N8" s="67"/>
+      <c r="O8" s="67"/>
+      <c r="P8" s="67"/>
+      <c r="Q8" s="67"/>
     </row>
     <row r="9" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="67" t="s">
+      <c r="D9" s="68" t="s">
         <v>107</v>
       </c>
-      <c r="E9" s="67"/>
-      <c r="F9" s="67"/>
-      <c r="G9" s="67"/>
+      <c r="E9" s="68"/>
+      <c r="F9" s="68"/>
+      <c r="G9" s="68"/>
       <c r="I9" s="3" t="s">
         <v>10</v>
       </c>
@@ -3052,12 +3021,12 @@
         <v>9</v>
       </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="68" t="s">
+      <c r="D10" s="69" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="69"/>
-      <c r="F10" s="69"/>
-      <c r="G10" s="69"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="70"/>
       <c r="I10" s="3" t="s">
         <v>47</v>
       </c>
@@ -3070,37 +3039,37 @@
         <v>9</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="68" t="s">
+      <c r="D11" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="E11" s="69"/>
-      <c r="F11" s="69"/>
-      <c r="G11" s="69"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="70"/>
+      <c r="G11" s="70"/>
       <c r="I11" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J11" s="2"/>
-      <c r="K11" s="64" t="s">
+      <c r="K11" s="65" t="s">
         <v>69</v>
       </c>
-      <c r="L11" s="64"/>
-      <c r="M11" s="64"/>
-      <c r="N11" s="64"/>
-      <c r="O11" s="64"/>
-      <c r="P11" s="64"/>
-      <c r="Q11" s="64"/>
+      <c r="L11" s="65"/>
+      <c r="M11" s="65"/>
+      <c r="N11" s="65"/>
+      <c r="O11" s="65"/>
+      <c r="P11" s="65"/>
+      <c r="Q11" s="65"/>
     </row>
     <row r="12" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="D12" s="68" t="s">
+      <c r="D12" s="69" t="s">
         <v>110</v>
       </c>
-      <c r="E12" s="69"/>
-      <c r="F12" s="69"/>
-      <c r="G12" s="69"/>
+      <c r="E12" s="70"/>
+      <c r="F12" s="70"/>
+      <c r="G12" s="70"/>
       <c r="I12" s="3"/>
       <c r="J12" s="2"/>
       <c r="K12" s="4"/>
@@ -3116,12 +3085,12 @@
         <v>9</v>
       </c>
       <c r="C13" s="2"/>
-      <c r="D13" s="68" t="s">
+      <c r="D13" s="69" t="s">
         <v>111</v>
       </c>
-      <c r="E13" s="69"/>
-      <c r="F13" s="69"/>
-      <c r="G13" s="69"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="70"/>
       <c r="I13" s="3"/>
       <c r="J13" s="2"/>
       <c r="K13" s="4"/>
@@ -3135,7 +3104,7 @@
     <row r="14" spans="2:22" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="34"/>
+      <c r="D14" s="26"/>
       <c r="I14" s="3"/>
       <c r="J14" s="2"/>
       <c r="K14" s="4"/>
@@ -3191,7 +3160,7 @@
       <c r="V15" s="9"/>
     </row>
     <row r="16" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="52">
+      <c r="B16" s="43">
         <v>1</v>
       </c>
       <c r="C16" s="11"/>
@@ -3201,7 +3170,7 @@
       <c r="E16" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="52" t="s">
+      <c r="F16" s="43" t="s">
         <v>82</v>
       </c>
       <c r="G16" s="13" t="s">
@@ -3210,23 +3179,23 @@
       <c r="H16" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="I16" s="52">
+      <c r="I16" s="43">
         <v>1</v>
       </c>
-      <c r="J16" s="52" t="s">
+      <c r="J16" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="L16" s="52" t="e">
+      <c r="L16" s="43" t="e">
         <f t="shared" ref="L16" si="0">F16*I16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N16" s="52" t="s">
+      <c r="N16" s="43" t="s">
         <v>85</v>
       </c>
-      <c r="O16" s="37" t="s">
+      <c r="O16" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="P16" s="37" t="e">
+      <c r="P16" s="28" t="e">
         <f t="shared" ref="P16" si="1">L16*O16</f>
         <v>#VALUE!</v>
       </c>
@@ -3236,7 +3205,7 @@
       <c r="V16" s="14"/>
     </row>
     <row r="17" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="52">
+      <c r="B17" s="43">
         <v>2</v>
       </c>
       <c r="C17" s="11"/>
@@ -3246,7 +3215,7 @@
       <c r="E17" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F17" s="52" t="s">
+      <c r="F17" s="43" t="s">
         <v>82</v>
       </c>
       <c r="G17" s="13" t="s">
@@ -3255,138 +3224,138 @@
       <c r="H17" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="I17" s="52">
+      <c r="I17" s="43">
         <v>1</v>
       </c>
-      <c r="J17" s="52" t="s">
+      <c r="J17" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="L17" s="52" t="e">
+      <c r="L17" s="43" t="e">
         <f t="shared" ref="L17:L19" si="2">F17*I17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N17" s="52" t="s">
+      <c r="N17" s="43" t="s">
         <v>85</v>
       </c>
-      <c r="O17" s="37" t="s">
+      <c r="O17" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="P17" s="37" t="e">
+      <c r="P17" s="28" t="e">
         <f t="shared" ref="P17:P19" si="3">L17*O17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Q17" s="82"/>
       <c r="R17" s="14"/>
       <c r="T17" s="14"/>
       <c r="U17" s="14"/>
       <c r="V17" s="14"/>
     </row>
     <row r="18" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="87">
+      <c r="B18" s="43">
         <v>3</v>
       </c>
-      <c r="C18" s="88"/>
-      <c r="D18" s="89" t="s">
+      <c r="C18" s="11"/>
+      <c r="D18" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="89" t="s">
+      <c r="E18" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="87" t="s">
+      <c r="F18" s="43" t="s">
         <v>82</v>
       </c>
-      <c r="G18" s="90" t="s">
+      <c r="G18" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="H18" s="82" t="s">
+      <c r="H18" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="I18" s="87">
+      <c r="I18" s="43">
         <v>1</v>
       </c>
-      <c r="J18" s="87" t="s">
+      <c r="J18" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="L18" s="52" t="e">
+      <c r="L18" s="43" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="N18" s="52" t="s">
+      <c r="N18" s="43" t="s">
         <v>85</v>
       </c>
-      <c r="O18" s="37" t="s">
+      <c r="O18" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="P18" s="37" t="e">
+      <c r="P18" s="28" t="e">
         <f t="shared" si="3"/>
         <v>#VALUE!</v>
       </c>
-      <c r="Q18" s="82"/>
       <c r="R18" s="14"/>
       <c r="T18" s="14"/>
       <c r="U18" s="14"/>
       <c r="V18" s="14"/>
     </row>
     <row r="19" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="87">
+      <c r="B19" s="43">
         <v>4</v>
       </c>
-      <c r="C19" s="88"/>
-      <c r="D19" s="89" t="s">
+      <c r="C19" s="11"/>
+      <c r="D19" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="E19" s="89" t="s">
+      <c r="E19" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="87" t="s">
+      <c r="F19" s="43" t="s">
         <v>82</v>
       </c>
-      <c r="G19" s="90" t="s">
+      <c r="G19" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="H19" s="82" t="s">
+      <c r="H19" s="72" t="s">
         <v>113</v>
       </c>
-      <c r="I19" s="87">
+      <c r="I19" s="73">
         <v>1</v>
       </c>
-      <c r="J19" s="87" t="s">
+      <c r="J19" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="L19" s="52" t="e">
+      <c r="K19" s="72"/>
+      <c r="L19" s="73" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
-      <c r="N19" s="52" t="s">
+      <c r="M19" s="72"/>
+      <c r="N19" s="73" t="s">
         <v>85</v>
       </c>
-      <c r="O19" s="37" t="s">
+      <c r="O19" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="P19" s="37" t="e">
+      <c r="P19" s="28" t="e">
         <f t="shared" si="3"/>
         <v>#VALUE!</v>
       </c>
-      <c r="Q19" s="82"/>
+      <c r="Q19" s="72"/>
       <c r="R19" s="14"/>
       <c r="T19" s="14"/>
       <c r="U19" s="14"/>
       <c r="V19" s="14"/>
     </row>
     <row r="20" spans="2:22" s="15" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="83"/>
-      <c r="C20" s="83"/>
-      <c r="D20" s="84"/>
-      <c r="E20" s="83"/>
-      <c r="F20" s="83"/>
-      <c r="G20" s="83"/>
-      <c r="H20" s="85"/>
-      <c r="I20" s="85" t="s">
+      <c r="B20" s="81"/>
+      <c r="C20" s="81"/>
+      <c r="D20" s="82"/>
+      <c r="E20" s="81"/>
+      <c r="F20" s="81"/>
+      <c r="G20" s="81"/>
+      <c r="H20" s="83"/>
+      <c r="I20" s="83" t="s">
         <v>49</v>
       </c>
-      <c r="J20" s="86"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="38" t="e">
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="29" t="e">
         <f>SUM(L16:L19)</f>
         <v>#VALUE!</v>
       </c>
@@ -3398,102 +3367,103 @@
       <c r="P20" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="Q20" s="83"/>
-    </row>
-    <row r="21" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="65" t="s">
+      <c r="Q20" s="81"/>
+    </row>
+    <row r="21" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="65"/>
-      <c r="D21" s="65"/>
-      <c r="E21" s="65"/>
-      <c r="F21" s="65"/>
-      <c r="G21" s="65"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="20" t="s">
+      <c r="C21" s="80"/>
+      <c r="D21" s="80"/>
+      <c r="E21" s="80"/>
+      <c r="F21" s="80"/>
+      <c r="G21" s="80"/>
+      <c r="H21" s="74"/>
+      <c r="I21" s="74" t="s">
         <v>41</v>
       </c>
-      <c r="J21" s="21"/>
-      <c r="K21" s="32"/>
-      <c r="L21" s="35">
+      <c r="J21" s="75"/>
+      <c r="K21" s="75"/>
+      <c r="L21" s="84">
         <v>0.15</v>
       </c>
-      <c r="M21" s="22"/>
-      <c r="N21" s="22"/>
-      <c r="O21" s="23"/>
-      <c r="P21" s="24" t="e">
+      <c r="M21" s="75"/>
+      <c r="N21" s="75"/>
+      <c r="O21" s="77"/>
+      <c r="P21" s="85" t="e">
         <f>-1*(L21*P20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Q21" s="83"/>
-    </row>
-    <row r="22" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="72" t="s">
+      <c r="Q21" s="76"/>
+    </row>
+    <row r="22" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="54" t="s">
         <v>115</v>
       </c>
-      <c r="C22" s="73"/>
-      <c r="D22" s="73"/>
-      <c r="E22" s="73"/>
-      <c r="F22" s="73"/>
-      <c r="G22" s="74"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3" t="s">
+      <c r="C22" s="55"/>
+      <c r="D22" s="55"/>
+      <c r="E22" s="55"/>
+      <c r="F22" s="55"/>
+      <c r="G22" s="56"/>
+      <c r="H22" s="78"/>
+      <c r="I22" s="78" t="s">
         <v>50</v>
       </c>
-      <c r="J22" s="19"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="25"/>
-      <c r="M22" s="26"/>
-      <c r="N22" s="26"/>
-      <c r="O22" s="26"/>
-      <c r="P22" s="27" t="s">
+      <c r="J22" s="76"/>
+      <c r="K22" s="76"/>
+      <c r="L22" s="20"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
+      <c r="O22" s="21"/>
+      <c r="P22" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="Q22" s="83"/>
+      <c r="Q22" s="76"/>
     </row>
     <row r="23" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="75"/>
-      <c r="C23" s="76"/>
-      <c r="D23" s="76"/>
-      <c r="E23" s="76"/>
-      <c r="F23" s="76"/>
-      <c r="G23" s="77"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
-      <c r="O23" s="19"/>
-      <c r="P23" s="19"/>
-      <c r="Q23" s="83"/>
+      <c r="B23" s="57"/>
+      <c r="C23" s="71"/>
+      <c r="D23" s="71"/>
+      <c r="E23" s="71"/>
+      <c r="F23" s="71"/>
+      <c r="G23" s="58"/>
+      <c r="H23" s="79"/>
+      <c r="I23" s="76"/>
+      <c r="J23" s="76"/>
+      <c r="K23" s="76"/>
+      <c r="L23" s="76"/>
+      <c r="M23" s="76"/>
+      <c r="N23" s="76"/>
+      <c r="O23" s="76"/>
+      <c r="P23" s="76"/>
+      <c r="Q23" s="76"/>
     </row>
     <row r="24" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="75"/>
-      <c r="C24" s="76"/>
-      <c r="D24" s="76"/>
-      <c r="E24" s="76"/>
-      <c r="F24" s="76"/>
-      <c r="G24" s="77"/>
+      <c r="B24" s="57"/>
+      <c r="C24" s="71"/>
+      <c r="D24" s="71"/>
+      <c r="E24" s="71"/>
+      <c r="F24" s="71"/>
+      <c r="G24" s="58"/>
       <c r="I24" s="3" t="s">
         <v>44</v>
       </c>
       <c r="J24" s="19"/>
       <c r="K24" s="19"/>
-      <c r="L24" s="36"/>
-      <c r="M24" s="36"/>
-      <c r="N24" s="36"/>
-      <c r="O24" s="36"/>
-      <c r="P24" s="36"/>
-      <c r="Q24" s="83"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="27"/>
+      <c r="Q24" s="19"/>
     </row>
     <row r="25" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="75"/>
-      <c r="C25" s="76"/>
-      <c r="D25" s="76"/>
-      <c r="E25" s="76"/>
-      <c r="F25" s="76"/>
-      <c r="G25" s="77"/>
+      <c r="B25" s="57"/>
+      <c r="C25" s="71"/>
+      <c r="D25" s="71"/>
+      <c r="E25" s="71"/>
+      <c r="F25" s="71"/>
+      <c r="G25" s="58"/>
       <c r="I25" s="3"/>
       <c r="J25" s="19"/>
       <c r="K25" s="19"/>
@@ -3502,90 +3472,90 @@
       <c r="N25" s="19"/>
       <c r="O25" s="19"/>
       <c r="P25" s="19"/>
-      <c r="Q25" s="83"/>
+      <c r="Q25" s="19"/>
     </row>
     <row r="26" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="75"/>
-      <c r="C26" s="76"/>
-      <c r="D26" s="76"/>
-      <c r="E26" s="76"/>
-      <c r="F26" s="76"/>
-      <c r="G26" s="77"/>
+      <c r="B26" s="57"/>
+      <c r="C26" s="71"/>
+      <c r="D26" s="71"/>
+      <c r="E26" s="71"/>
+      <c r="F26" s="71"/>
+      <c r="G26" s="58"/>
       <c r="I26" s="3" t="s">
         <v>43</v>
       </c>
       <c r="J26" s="19"/>
       <c r="K26" s="19"/>
-      <c r="L26" s="36"/>
-      <c r="M26" s="36"/>
-      <c r="N26" s="36"/>
-      <c r="O26" s="36"/>
-      <c r="P26" s="36"/>
-      <c r="Q26" s="83"/>
+      <c r="L26" s="27"/>
+      <c r="M26" s="27"/>
+      <c r="N26" s="27"/>
+      <c r="O26" s="27"/>
+      <c r="P26" s="27"/>
+      <c r="Q26" s="19"/>
     </row>
     <row r="27" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="78"/>
-      <c r="C27" s="79"/>
-      <c r="D27" s="79"/>
-      <c r="E27" s="79"/>
-      <c r="F27" s="79"/>
-      <c r="G27" s="80"/>
-      <c r="I27" s="30"/>
-      <c r="J27" s="30"/>
-      <c r="K27" s="30"/>
-      <c r="L27" s="30"/>
-      <c r="M27" s="30"/>
-      <c r="N27" s="30"/>
-      <c r="O27" s="30"/>
-      <c r="P27" s="30"/>
-      <c r="Q27" s="83"/>
+      <c r="B27" s="59"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="60"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="60"/>
+      <c r="G27" s="61"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="25"/>
+      <c r="M27" s="25"/>
+      <c r="N27" s="25"/>
+      <c r="O27" s="25"/>
+      <c r="P27" s="25"/>
+      <c r="Q27" s="19"/>
     </row>
     <row r="28" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I28" s="30"/>
-      <c r="J28" s="30"/>
-      <c r="K28" s="30"/>
-      <c r="L28" s="30"/>
-      <c r="M28" s="30"/>
-      <c r="N28" s="30"/>
-      <c r="O28" s="30"/>
-      <c r="P28" s="30"/>
-      <c r="Q28" s="83"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="25"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="25"/>
+      <c r="M28" s="25"/>
+      <c r="N28" s="25"/>
+      <c r="O28" s="25"/>
+      <c r="P28" s="25"/>
+      <c r="Q28" s="19"/>
     </row>
     <row r="29" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="81" t="s">
+      <c r="B29" s="62" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="81"/>
-      <c r="D29" s="81"/>
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
-      <c r="G29" s="40"/>
-      <c r="I29" s="30"/>
-      <c r="J29" s="30"/>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
-      <c r="N29" s="30"/>
-      <c r="O29" s="30"/>
-      <c r="P29" s="30"/>
-      <c r="Q29" s="83"/>
+      <c r="C29" s="62"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="25"/>
+      <c r="K29" s="25"/>
+      <c r="L29" s="25"/>
+      <c r="M29" s="25"/>
+      <c r="N29" s="25"/>
+      <c r="O29" s="25"/>
+      <c r="P29" s="25"/>
+      <c r="Q29" s="19"/>
     </row>
     <row r="30" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
-      <c r="E30" s="40"/>
-      <c r="F30" s="40"/>
-      <c r="G30" s="40"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="30"/>
-      <c r="K30" s="30"/>
-      <c r="L30" s="30"/>
-      <c r="M30" s="30"/>
-      <c r="N30" s="30"/>
-      <c r="O30" s="30"/>
-      <c r="P30" s="30"/>
-      <c r="Q30" s="83"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="25"/>
+      <c r="K30" s="25"/>
+      <c r="L30" s="25"/>
+      <c r="M30" s="25"/>
+      <c r="N30" s="25"/>
+      <c r="O30" s="25"/>
+      <c r="P30" s="25"/>
+      <c r="Q30" s="19"/>
     </row>
     <row r="31" spans="2:22" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
@@ -3600,48 +3570,48 @@
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
-      <c r="I31" s="30"/>
-      <c r="J31" s="30"/>
-      <c r="K31" s="30"/>
-      <c r="L31" s="30"/>
-      <c r="M31" s="30"/>
-      <c r="N31" s="30"/>
-      <c r="O31" s="30"/>
-      <c r="P31" s="30"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="25"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="25"/>
+      <c r="M31" s="25"/>
+      <c r="N31" s="25"/>
+      <c r="O31" s="25"/>
+      <c r="P31" s="25"/>
       <c r="Q31" s="19"/>
     </row>
     <row r="32" spans="2:22" s="18" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="41" t="s">
+      <c r="B32" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="41"/>
-      <c r="D32" s="42">
+      <c r="C32" s="32"/>
+      <c r="D32" s="33">
         <v>700</v>
       </c>
-      <c r="E32" s="44">
+      <c r="E32" s="35">
         <f>D32*0.85</f>
         <v>595</v>
       </c>
-      <c r="I32" s="30"/>
-      <c r="J32" s="30"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="30"/>
-      <c r="M32" s="30"/>
-      <c r="N32" s="30"/>
-      <c r="O32" s="30"/>
-      <c r="P32" s="30"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="25"/>
+      <c r="K32" s="25"/>
+      <c r="L32" s="25"/>
+      <c r="M32" s="25"/>
+      <c r="N32" s="25"/>
+      <c r="O32" s="25"/>
+      <c r="P32" s="25"/>
       <c r="Q32" s="19"/>
     </row>
     <row r="33" spans="2:17" s="18" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="45" t="s">
+      <c r="B33" s="36" t="s">
         <v>55</v>
       </c>
       <c r="C33" s="19"/>
-      <c r="D33" s="43">
+      <c r="D33" s="34">
         <f>SUM(D32:D32)</f>
         <v>700</v>
       </c>
-      <c r="E33" s="46">
+      <c r="E33" s="37">
         <f>SUM(E32:E32)</f>
         <v>595</v>
       </c>
@@ -3715,6 +3685,9 @@
     </dataRefs>
   </dataConsolidate>
   <mergeCells count="19">
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="D13:G13"/>
     <mergeCell ref="B22:G27"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="F1:L1"/>
@@ -3731,9 +3704,6 @@
     <mergeCell ref="L6:Q6"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="D10:G10"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="D13:G13"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <hyperlinks>
@@ -3769,9 +3739,9 @@
     <col min="16" max="16" width="12.5703125" customWidth="1"/>
     <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="11" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.7109375" style="49" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.7109375" style="40" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="30" style="54" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="30" style="45" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -3837,13 +3807,13 @@
       <c r="R1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="S1" s="48" t="s">
+      <c r="S1" s="39" t="s">
         <v>56</v>
       </c>
       <c r="T1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="U1" s="53" t="s">
+      <c r="U1" s="44" t="s">
         <v>65</v>
       </c>
       <c r="V1" s="9" t="s">
@@ -3864,7 +3834,7 @@
       <c r="AA1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AB1" s="53" t="s">
+      <c r="AB1" s="44" t="s">
         <v>66</v>
       </c>
       <c r="AC1" s="5" t="s">
@@ -3875,29 +3845,29 @@
       <c r="A2" t="s">
         <v>101</v>
       </c>
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="39" t="str">
+      <c r="C2" s="30" t="str">
         <f t="shared" ref="C2" si="0">B2</f>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D2" s="56" t="s">
+      <c r="D2" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E2" s="57" t="s">
+      <c r="E2" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F2" s="57" t="s">
+      <c r="F2" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="57" t="s">
+      <c r="G2" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H2" t="s">
         <v>89</v>
       </c>
-      <c r="I2" s="58" t="s">
+      <c r="I2" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J2" t="s">
@@ -3915,22 +3885,22 @@
       <c r="O2" t="s">
         <v>78</v>
       </c>
-      <c r="P2" s="59" t="s">
+      <c r="P2" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R2" s="59" t="s">
+      <c r="R2" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S2" s="60" t="s">
+      <c r="S2" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T2" s="59" t="s">
+      <c r="T2" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U2" s="61" t="s">
+      <c r="U2" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V2" s="59" t="s">
+      <c r="V2" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W2" t="s">
@@ -3948,7 +3918,7 @@
       <c r="AA2" t="s">
         <v>99</v>
       </c>
-      <c r="AB2" s="61" t="s">
+      <c r="AB2" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC2" t="s">
@@ -3959,29 +3929,29 @@
       <c r="A3" t="s">
         <v>101</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="39" t="str">
+      <c r="C3" s="30" t="str">
         <f t="shared" ref="C3:C13" si="1">B3</f>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D3" s="56" t="s">
+      <c r="D3" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E3" s="57" t="s">
+      <c r="E3" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F3" s="57" t="s">
+      <c r="F3" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G3" s="57" t="s">
+      <c r="G3" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H3" t="s">
         <v>89</v>
       </c>
-      <c r="I3" s="58" t="s">
+      <c r="I3" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J3" t="s">
@@ -3999,22 +3969,22 @@
       <c r="O3" t="s">
         <v>78</v>
       </c>
-      <c r="P3" s="59" t="s">
+      <c r="P3" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R3" s="59" t="s">
+      <c r="R3" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S3" s="60" t="s">
+      <c r="S3" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T3" s="59" t="s">
+      <c r="T3" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U3" s="61" t="s">
+      <c r="U3" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V3" s="59" t="s">
+      <c r="V3" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W3" t="s">
@@ -4032,7 +4002,7 @@
       <c r="AA3" t="s">
         <v>99</v>
       </c>
-      <c r="AB3" s="61" t="s">
+      <c r="AB3" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC3" t="s">
@@ -4043,29 +4013,29 @@
       <c r="A4" t="s">
         <v>101</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C4" s="39" t="str">
+      <c r="C4" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D4" s="56" t="s">
+      <c r="D4" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E4" s="57" t="s">
+      <c r="E4" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F4" s="57" t="s">
+      <c r="F4" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G4" s="57" t="s">
+      <c r="G4" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H4" t="s">
         <v>89</v>
       </c>
-      <c r="I4" s="58" t="s">
+      <c r="I4" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J4" t="s">
@@ -4083,22 +4053,22 @@
       <c r="O4" t="s">
         <v>78</v>
       </c>
-      <c r="P4" s="59" t="s">
+      <c r="P4" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R4" s="59" t="s">
+      <c r="R4" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S4" s="60" t="s">
+      <c r="S4" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T4" s="59" t="s">
+      <c r="T4" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U4" s="61" t="s">
+      <c r="U4" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V4" s="59" t="s">
+      <c r="V4" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W4" t="s">
@@ -4116,7 +4086,7 @@
       <c r="AA4" t="s">
         <v>99</v>
       </c>
-      <c r="AB4" s="61" t="s">
+      <c r="AB4" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC4" t="s">
@@ -4127,29 +4097,29 @@
       <c r="A5" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="39" t="str">
+      <c r="C5" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D5" s="56" t="s">
+      <c r="D5" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E5" s="57" t="s">
+      <c r="E5" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="57" t="s">
+      <c r="F5" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G5" s="57" t="s">
+      <c r="G5" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H5" t="s">
         <v>89</v>
       </c>
-      <c r="I5" s="58" t="s">
+      <c r="I5" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J5" t="s">
@@ -4167,22 +4137,22 @@
       <c r="O5" t="s">
         <v>78</v>
       </c>
-      <c r="P5" s="59" t="s">
+      <c r="P5" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R5" s="59" t="s">
+      <c r="R5" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S5" s="60" t="s">
+      <c r="S5" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T5" s="59" t="s">
+      <c r="T5" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U5" s="61" t="s">
+      <c r="U5" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V5" s="59" t="s">
+      <c r="V5" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W5" t="s">
@@ -4200,7 +4170,7 @@
       <c r="AA5" t="s">
         <v>99</v>
       </c>
-      <c r="AB5" s="61" t="s">
+      <c r="AB5" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC5" t="s">
@@ -4211,29 +4181,29 @@
       <c r="A6" t="s">
         <v>101</v>
       </c>
-      <c r="B6" s="55" t="s">
+      <c r="B6" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="39" t="str">
+      <c r="C6" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D6" s="56" t="s">
+      <c r="D6" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E6" s="57" t="s">
+      <c r="E6" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="57" t="s">
+      <c r="F6" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G6" s="57" t="s">
+      <c r="G6" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H6" t="s">
         <v>89</v>
       </c>
-      <c r="I6" s="58" t="s">
+      <c r="I6" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J6" t="s">
@@ -4251,22 +4221,22 @@
       <c r="O6" t="s">
         <v>78</v>
       </c>
-      <c r="P6" s="59" t="s">
+      <c r="P6" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R6" s="59" t="s">
+      <c r="R6" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S6" s="60" t="s">
+      <c r="S6" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T6" s="59" t="s">
+      <c r="T6" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U6" s="61" t="s">
+      <c r="U6" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V6" s="59" t="s">
+      <c r="V6" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W6" t="s">
@@ -4284,7 +4254,7 @@
       <c r="AA6" t="s">
         <v>99</v>
       </c>
-      <c r="AB6" s="61" t="s">
+      <c r="AB6" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC6" t="s">
@@ -4295,29 +4265,29 @@
       <c r="A7" t="s">
         <v>101</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="B7" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C7" s="39" t="str">
+      <c r="C7" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D7" s="56" t="s">
+      <c r="D7" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E7" s="57" t="s">
+      <c r="E7" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F7" s="57" t="s">
+      <c r="F7" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G7" s="57" t="s">
+      <c r="G7" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H7" t="s">
         <v>89</v>
       </c>
-      <c r="I7" s="58" t="s">
+      <c r="I7" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J7" t="s">
@@ -4335,22 +4305,22 @@
       <c r="O7" t="s">
         <v>78</v>
       </c>
-      <c r="P7" s="59" t="s">
+      <c r="P7" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R7" s="59" t="s">
+      <c r="R7" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S7" s="60" t="s">
+      <c r="S7" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T7" s="59" t="s">
+      <c r="T7" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U7" s="61" t="s">
+      <c r="U7" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V7" s="59" t="s">
+      <c r="V7" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W7" t="s">
@@ -4368,7 +4338,7 @@
       <c r="AA7" t="s">
         <v>99</v>
       </c>
-      <c r="AB7" s="61" t="s">
+      <c r="AB7" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC7" t="s">
@@ -4379,29 +4349,29 @@
       <c r="A8" t="s">
         <v>101</v>
       </c>
-      <c r="B8" s="55" t="s">
+      <c r="B8" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="39" t="str">
+      <c r="C8" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D8" s="56" t="s">
+      <c r="D8" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E8" s="57" t="s">
+      <c r="E8" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F8" s="57" t="s">
+      <c r="F8" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G8" s="57" t="s">
+      <c r="G8" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H8" t="s">
         <v>89</v>
       </c>
-      <c r="I8" s="58" t="s">
+      <c r="I8" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J8" t="s">
@@ -4419,22 +4389,22 @@
       <c r="O8" t="s">
         <v>78</v>
       </c>
-      <c r="P8" s="59" t="s">
+      <c r="P8" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R8" s="59" t="s">
+      <c r="R8" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S8" s="60" t="s">
+      <c r="S8" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T8" s="59" t="s">
+      <c r="T8" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U8" s="61" t="s">
+      <c r="U8" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V8" s="59" t="s">
+      <c r="V8" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W8" t="s">
@@ -4452,7 +4422,7 @@
       <c r="AA8" t="s">
         <v>99</v>
       </c>
-      <c r="AB8" s="61" t="s">
+      <c r="AB8" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC8" t="s">
@@ -4463,29 +4433,29 @@
       <c r="A9" t="s">
         <v>101</v>
       </c>
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C9" s="39" t="str">
+      <c r="C9" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D9" s="56" t="s">
+      <c r="D9" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E9" s="57" t="s">
+      <c r="E9" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F9" s="57" t="s">
+      <c r="F9" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G9" s="57" t="s">
+      <c r="G9" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H9" t="s">
         <v>89</v>
       </c>
-      <c r="I9" s="58" t="s">
+      <c r="I9" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J9" t="s">
@@ -4503,22 +4473,22 @@
       <c r="O9" t="s">
         <v>78</v>
       </c>
-      <c r="P9" s="59" t="s">
+      <c r="P9" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R9" s="59" t="s">
+      <c r="R9" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S9" s="60" t="s">
+      <c r="S9" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T9" s="59" t="s">
+      <c r="T9" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U9" s="61" t="s">
+      <c r="U9" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V9" s="59" t="s">
+      <c r="V9" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W9" t="s">
@@ -4536,7 +4506,7 @@
       <c r="AA9" t="s">
         <v>99</v>
       </c>
-      <c r="AB9" s="61" t="s">
+      <c r="AB9" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC9" t="s">
@@ -4547,29 +4517,29 @@
       <c r="A10" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="55" t="s">
+      <c r="B10" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="39" t="str">
+      <c r="C10" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D10" s="56" t="s">
+      <c r="D10" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E10" s="57" t="s">
+      <c r="E10" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="57" t="s">
+      <c r="F10" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G10" s="57" t="s">
+      <c r="G10" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H10" t="s">
         <v>89</v>
       </c>
-      <c r="I10" s="58" t="s">
+      <c r="I10" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J10" t="s">
@@ -4587,22 +4557,22 @@
       <c r="O10" t="s">
         <v>78</v>
       </c>
-      <c r="P10" s="59" t="s">
+      <c r="P10" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R10" s="59" t="s">
+      <c r="R10" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S10" s="60" t="s">
+      <c r="S10" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T10" s="59" t="s">
+      <c r="T10" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U10" s="61" t="s">
+      <c r="U10" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V10" s="59" t="s">
+      <c r="V10" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W10" t="s">
@@ -4620,7 +4590,7 @@
       <c r="AA10" t="s">
         <v>99</v>
       </c>
-      <c r="AB10" s="61" t="s">
+      <c r="AB10" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC10" t="s">
@@ -4631,29 +4601,29 @@
       <c r="A11" t="s">
         <v>101</v>
       </c>
-      <c r="B11" s="55" t="s">
+      <c r="B11" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C11" s="39" t="str">
+      <c r="C11" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D11" s="56" t="s">
+      <c r="D11" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E11" s="57" t="s">
+      <c r="E11" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F11" s="57" t="s">
+      <c r="F11" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G11" s="57" t="s">
+      <c r="G11" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H11" t="s">
         <v>89</v>
       </c>
-      <c r="I11" s="58" t="s">
+      <c r="I11" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J11" t="s">
@@ -4671,22 +4641,22 @@
       <c r="O11" t="s">
         <v>78</v>
       </c>
-      <c r="P11" s="59" t="s">
+      <c r="P11" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R11" s="59" t="s">
+      <c r="R11" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S11" s="60" t="s">
+      <c r="S11" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T11" s="59" t="s">
+      <c r="T11" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U11" s="61" t="s">
+      <c r="U11" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V11" s="59" t="s">
+      <c r="V11" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W11" t="s">
@@ -4704,7 +4674,7 @@
       <c r="AA11" t="s">
         <v>99</v>
       </c>
-      <c r="AB11" s="61" t="s">
+      <c r="AB11" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC11" t="s">
@@ -4715,29 +4685,29 @@
       <c r="A12" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="55" t="s">
+      <c r="B12" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C12" s="39" t="str">
+      <c r="C12" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D12" s="56" t="s">
+      <c r="D12" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E12" s="57" t="s">
+      <c r="E12" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F12" s="57" t="s">
+      <c r="F12" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G12" s="57" t="s">
+      <c r="G12" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H12" t="s">
         <v>89</v>
       </c>
-      <c r="I12" s="58" t="s">
+      <c r="I12" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J12" t="s">
@@ -4755,22 +4725,22 @@
       <c r="O12" t="s">
         <v>78</v>
       </c>
-      <c r="P12" s="59" t="s">
+      <c r="P12" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R12" s="59" t="s">
+      <c r="R12" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S12" s="60" t="s">
+      <c r="S12" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T12" s="59" t="s">
+      <c r="T12" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U12" s="61" t="s">
+      <c r="U12" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V12" s="59" t="s">
+      <c r="V12" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W12" t="s">
@@ -4788,7 +4758,7 @@
       <c r="AA12" t="s">
         <v>99</v>
       </c>
-      <c r="AB12" s="61" t="s">
+      <c r="AB12" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC12" t="s">
@@ -4799,29 +4769,29 @@
       <c r="A13" t="s">
         <v>101</v>
       </c>
-      <c r="B13" s="55" t="s">
+      <c r="B13" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="C13" s="39" t="str">
+      <c r="C13" s="30" t="str">
         <f t="shared" si="1"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D13" s="56" t="s">
+      <c r="D13" s="47" t="s">
         <v>103</v>
       </c>
-      <c r="E13" s="57" t="s">
+      <c r="E13" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="F13" s="57" t="s">
+      <c r="F13" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="G13" s="57" t="s">
+      <c r="G13" s="48" t="s">
         <v>85</v>
       </c>
       <c r="H13" t="s">
         <v>89</v>
       </c>
-      <c r="I13" s="58" t="s">
+      <c r="I13" s="49" t="s">
         <v>90</v>
       </c>
       <c r="J13" t="s">
@@ -4839,22 +4809,22 @@
       <c r="O13" t="s">
         <v>78</v>
       </c>
-      <c r="P13" s="59" t="s">
+      <c r="P13" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="R13" s="59" t="s">
+      <c r="R13" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="S13" s="60" t="s">
+      <c r="S13" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="T13" s="59" t="s">
+      <c r="T13" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="U13" s="61" t="s">
+      <c r="U13" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="V13" s="59" t="s">
+      <c r="V13" s="50" t="s">
         <v>96</v>
       </c>
       <c r="W13" t="s">
@@ -4872,7 +4842,7 @@
       <c r="AA13" t="s">
         <v>99</v>
       </c>
-      <c r="AB13" s="61" t="s">
+      <c r="AB13" s="52" t="s">
         <v>70</v>
       </c>
       <c r="AC13" t="s">
@@ -4880,196 +4850,196 @@
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B14" s="55"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="57"/>
-      <c r="G14" s="57"/>
-      <c r="I14" s="58"/>
-      <c r="P14" s="62"/>
-      <c r="R14" s="62"/>
-      <c r="S14" s="60"/>
-      <c r="T14" s="62"/>
-      <c r="U14" s="61"/>
-      <c r="V14" s="62"/>
-      <c r="AB14" s="61"/>
+      <c r="B14" s="46"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="I14" s="49"/>
+      <c r="P14" s="53"/>
+      <c r="R14" s="53"/>
+      <c r="S14" s="51"/>
+      <c r="T14" s="53"/>
+      <c r="U14" s="52"/>
+      <c r="V14" s="53"/>
+      <c r="AB14" s="52"/>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B15" s="55"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="56"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="57"/>
-      <c r="G15" s="57"/>
-      <c r="I15" s="58"/>
-      <c r="P15" s="62"/>
-      <c r="R15" s="62"/>
-      <c r="S15" s="60"/>
-      <c r="T15" s="62"/>
-      <c r="U15" s="61"/>
-      <c r="V15" s="62"/>
-      <c r="AB15" s="61"/>
+      <c r="B15" s="46"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="I15" s="49"/>
+      <c r="P15" s="53"/>
+      <c r="R15" s="53"/>
+      <c r="S15" s="51"/>
+      <c r="T15" s="53"/>
+      <c r="U15" s="52"/>
+      <c r="V15" s="53"/>
+      <c r="AB15" s="52"/>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B16" s="55"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="56"/>
-      <c r="E16" s="57"/>
-      <c r="F16" s="57"/>
-      <c r="G16" s="57"/>
-      <c r="I16" s="58"/>
-      <c r="P16" s="62"/>
-      <c r="R16" s="62"/>
-      <c r="S16" s="60"/>
-      <c r="T16" s="62"/>
-      <c r="U16" s="61"/>
-      <c r="V16" s="62"/>
-      <c r="AB16" s="61"/>
+      <c r="B16" s="46"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="48"/>
+      <c r="I16" s="49"/>
+      <c r="P16" s="53"/>
+      <c r="R16" s="53"/>
+      <c r="S16" s="51"/>
+      <c r="T16" s="53"/>
+      <c r="U16" s="52"/>
+      <c r="V16" s="53"/>
+      <c r="AB16" s="52"/>
     </row>
     <row r="17" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B17" s="55"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="57"/>
-      <c r="F17" s="57"/>
-      <c r="G17" s="57"/>
-      <c r="I17" s="58"/>
-      <c r="P17" s="62"/>
-      <c r="R17" s="62"/>
-      <c r="S17" s="60"/>
-      <c r="T17" s="62"/>
-      <c r="U17" s="61"/>
-      <c r="V17" s="62"/>
-      <c r="AB17" s="61"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="48"/>
+      <c r="I17" s="49"/>
+      <c r="P17" s="53"/>
+      <c r="R17" s="53"/>
+      <c r="S17" s="51"/>
+      <c r="T17" s="53"/>
+      <c r="U17" s="52"/>
+      <c r="V17" s="53"/>
+      <c r="AB17" s="52"/>
     </row>
     <row r="18" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B18" s="55"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="56"/>
-      <c r="E18" s="57"/>
-      <c r="F18" s="57"/>
-      <c r="G18" s="57"/>
-      <c r="I18" s="58"/>
-      <c r="P18" s="62"/>
-      <c r="R18" s="62"/>
-      <c r="S18" s="60"/>
-      <c r="T18" s="62"/>
-      <c r="U18" s="61"/>
-      <c r="V18" s="62"/>
-      <c r="AB18" s="61"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="48"/>
+      <c r="I18" s="49"/>
+      <c r="P18" s="53"/>
+      <c r="R18" s="53"/>
+      <c r="S18" s="51"/>
+      <c r="T18" s="53"/>
+      <c r="U18" s="52"/>
+      <c r="V18" s="53"/>
+      <c r="AB18" s="52"/>
     </row>
     <row r="19" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B19" s="55"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="57"/>
-      <c r="G19" s="57"/>
-      <c r="I19" s="58"/>
-      <c r="P19" s="62"/>
-      <c r="R19" s="62"/>
-      <c r="S19" s="60"/>
-      <c r="T19" s="62"/>
-      <c r="U19" s="61"/>
-      <c r="V19" s="62"/>
-      <c r="AB19" s="61"/>
+      <c r="B19" s="46"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="48"/>
+      <c r="I19" s="49"/>
+      <c r="P19" s="53"/>
+      <c r="R19" s="53"/>
+      <c r="S19" s="51"/>
+      <c r="T19" s="53"/>
+      <c r="U19" s="52"/>
+      <c r="V19" s="53"/>
+      <c r="AB19" s="52"/>
     </row>
     <row r="20" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B20" s="55"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="56"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
-      <c r="I20" s="58"/>
-      <c r="P20" s="62"/>
-      <c r="R20" s="62"/>
-      <c r="S20" s="60"/>
-      <c r="T20" s="62"/>
-      <c r="U20" s="61"/>
-      <c r="V20" s="62"/>
-      <c r="AB20" s="61"/>
+      <c r="B20" s="46"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="48"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="48"/>
+      <c r="I20" s="49"/>
+      <c r="P20" s="53"/>
+      <c r="R20" s="53"/>
+      <c r="S20" s="51"/>
+      <c r="T20" s="53"/>
+      <c r="U20" s="52"/>
+      <c r="V20" s="53"/>
+      <c r="AB20" s="52"/>
     </row>
     <row r="21" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B21" s="55"/>
-      <c r="C21" s="39"/>
-      <c r="D21" s="56"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="57"/>
-      <c r="G21" s="57"/>
-      <c r="I21" s="58"/>
-      <c r="P21" s="62"/>
-      <c r="R21" s="62"/>
-      <c r="S21" s="60"/>
-      <c r="T21" s="62"/>
-      <c r="U21" s="61"/>
-      <c r="V21" s="62"/>
-      <c r="AB21" s="61"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="47"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="48"/>
+      <c r="I21" s="49"/>
+      <c r="P21" s="53"/>
+      <c r="R21" s="53"/>
+      <c r="S21" s="51"/>
+      <c r="T21" s="53"/>
+      <c r="U21" s="52"/>
+      <c r="V21" s="53"/>
+      <c r="AB21" s="52"/>
     </row>
     <row r="22" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B22" s="55"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="56"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
-      <c r="I22" s="58"/>
-      <c r="P22" s="62"/>
-      <c r="R22" s="62"/>
-      <c r="S22" s="60"/>
-      <c r="T22" s="62"/>
-      <c r="U22" s="61"/>
-      <c r="V22" s="62"/>
-      <c r="AB22" s="61"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="47"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48"/>
+      <c r="I22" s="49"/>
+      <c r="P22" s="53"/>
+      <c r="R22" s="53"/>
+      <c r="S22" s="51"/>
+      <c r="T22" s="53"/>
+      <c r="U22" s="52"/>
+      <c r="V22" s="53"/>
+      <c r="AB22" s="52"/>
     </row>
     <row r="23" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B23" s="55"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="I23" s="58"/>
-      <c r="P23" s="62"/>
-      <c r="R23" s="62"/>
-      <c r="S23" s="60"/>
-      <c r="T23" s="62"/>
-      <c r="U23" s="61"/>
-      <c r="V23" s="62"/>
-      <c r="AB23" s="61"/>
+      <c r="B23" s="46"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="47"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="I23" s="49"/>
+      <c r="P23" s="53"/>
+      <c r="R23" s="53"/>
+      <c r="S23" s="51"/>
+      <c r="T23" s="53"/>
+      <c r="U23" s="52"/>
+      <c r="V23" s="53"/>
+      <c r="AB23" s="52"/>
     </row>
     <row r="24" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B24" s="55"/>
-      <c r="C24" s="39"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="57"/>
-      <c r="F24" s="57"/>
-      <c r="G24" s="57"/>
-      <c r="I24" s="58"/>
-      <c r="P24" s="62"/>
-      <c r="R24" s="62"/>
-      <c r="S24" s="60"/>
-      <c r="T24" s="62"/>
-      <c r="U24" s="61"/>
-      <c r="V24" s="62"/>
-      <c r="AB24" s="61"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="47"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="I24" s="49"/>
+      <c r="P24" s="53"/>
+      <c r="R24" s="53"/>
+      <c r="S24" s="51"/>
+      <c r="T24" s="53"/>
+      <c r="U24" s="52"/>
+      <c r="V24" s="53"/>
+      <c r="AB24" s="52"/>
     </row>
     <row r="25" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B25" s="55"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="57"/>
-      <c r="F25" s="57"/>
-      <c r="G25" s="57"/>
-      <c r="I25" s="58"/>
-      <c r="P25" s="62"/>
-      <c r="R25" s="62"/>
-      <c r="S25" s="60"/>
-      <c r="T25" s="62"/>
-      <c r="U25" s="61"/>
-      <c r="V25" s="62"/>
-      <c r="AB25" s="61"/>
+      <c r="B25" s="46"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="47"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
+      <c r="I25" s="49"/>
+      <c r="P25" s="53"/>
+      <c r="R25" s="53"/>
+      <c r="S25" s="51"/>
+      <c r="T25" s="53"/>
+      <c r="U25" s="52"/>
+      <c r="V25" s="53"/>
+      <c r="AB25" s="52"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AC1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
@@ -5090,7 +5060,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="41" t="s">
         <v>60</v>
       </c>
       <c r="B3" t="s">
@@ -5104,17 +5074,17 @@
       <c r="A4" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="C4" s="51"/>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B5" s="51">
+      <c r="B5" s="42">
         <v>0</v>
       </c>
-      <c r="C5" s="51">
+      <c r="C5" s="42">
         <v>0</v>
       </c>
     </row>
@@ -5122,10 +5092,10 @@
       <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="51">
+      <c r="B6" s="42">
         <v>0</v>
       </c>
-      <c r="C6" s="51">
+      <c r="C6" s="42">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Backwrite: fix row height inconsistency causing black line between items 4-5
_snapshot_row now captures the source row's height, and _apply_snapshot
restores it on every cloned row. Template rows 16-19 have height=18.75;
without this fix cloned rows 20+ defaulted to 15.0, producing a visible
height-change line at the boundary of the 4th and 5th line items.

Also restores the thick top border on template row 20 that was accidentally
removed in the previous attempt, which is the top edge of the Gross Amount
box sitting below the last data row.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/backwrite/template.xlsx
+++ b/src/backwrite/template.xlsx
@@ -332,7 +332,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -642,6 +642,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick"/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thick"/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick"/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -737,7 +759,7 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1004,6 +1026,24 @@
     </xf>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="89">
@@ -2543,7 +2583,7 @@
     <col hidden="1" width="7.140625" customWidth="1" style="23" min="26" max="26"/>
     <col hidden="1" width="8.42578125" customWidth="1" style="23" min="27" max="28"/>
     <col hidden="1" width="6.42578125" customWidth="1" style="23" min="29" max="29"/>
-    <col hidden="1" style="23" min="30" max="36"/>
+    <col hidden="1" width="13" customWidth="1" style="23" min="30" max="36"/>
     <col hidden="1" width="149.140625" customWidth="1" style="23" min="37" max="16384"/>
   </cols>
   <sheetData>
@@ -3194,37 +3234,37 @@
       <c r="V19" s="92" t="n"/>
     </row>
     <row r="20" ht="15" customFormat="1" customHeight="1" s="15" thickTop="1">
-      <c r="B20" s="76" t="n"/>
-      <c r="C20" s="76" t="n"/>
-      <c r="D20" s="62" t="n"/>
-      <c r="E20" s="76" t="n"/>
-      <c r="F20" s="76" t="n"/>
-      <c r="G20" s="76" t="n"/>
-      <c r="H20" s="74" t="n"/>
-      <c r="I20" s="74" t="inlineStr">
+      <c r="B20" s="110" t="n"/>
+      <c r="C20" s="110" t="n"/>
+      <c r="D20" s="111" t="n"/>
+      <c r="E20" s="110" t="n"/>
+      <c r="F20" s="110" t="n"/>
+      <c r="G20" s="110" t="n"/>
+      <c r="H20" s="112" t="n"/>
+      <c r="I20" s="112" t="inlineStr">
         <is>
           <t>Gross Amount</t>
         </is>
       </c>
-      <c r="J20" s="75" t="n"/>
-      <c r="K20" s="75" t="n"/>
-      <c r="L20" s="93">
+      <c r="J20" s="113" t="n"/>
+      <c r="K20" s="113" t="n"/>
+      <c r="L20" s="114">
         <f>SUM(L16:L19)</f>
         <v/>
       </c>
-      <c r="M20" s="75" t="n"/>
-      <c r="N20" s="75" t="inlineStr">
+      <c r="M20" s="113" t="n"/>
+      <c r="N20" s="113" t="inlineStr">
         <is>
           <t>spots</t>
         </is>
       </c>
-      <c r="O20" s="75" t="n"/>
-      <c r="P20" s="94" t="inlineStr">
+      <c r="O20" s="113" t="n"/>
+      <c r="P20" s="115" t="inlineStr">
         <is>
           <t>&lt;total_gross&gt;</t>
         </is>
       </c>
-      <c r="Q20" s="76" t="n"/>
+      <c r="Q20" s="110" t="n"/>
     </row>
     <row r="21" ht="15" customFormat="1" customHeight="1" s="79">
       <c r="B21" s="80" t="inlineStr">

</xml_diff>

<commit_message>
Backwrite: fix Q-column black line and monthly breakdown double border
Template: remove thick top from Q20 (the Gross Amount box separator now ends
at column P, not Q, so no stray line bleeds into the empty column).

Template: remove bottom=double from monthly data row 32 so cloned month rows
don't all inherit the double underline.

Code (_fill_monthly_breakdown): apply bottom=double only to the last filled
data row, producing a single separator between the month rows and Total.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/backwrite/template.xlsx
+++ b/src/backwrite/template.xlsx
@@ -332,7 +332,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -664,6 +664,12 @@
       <top style="thick"/>
       <bottom/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -759,7 +765,7 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1045,6 +1051,12 @@
     <xf numFmtId="165" fontId="9" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="55"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="89">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3264,7 +3276,7 @@
           <t>&lt;total_gross&gt;</t>
         </is>
       </c>
-      <c r="Q20" s="110" t="n"/>
+      <c r="Q20" s="116" t="n"/>
     </row>
     <row r="21" ht="15" customFormat="1" customHeight="1" s="79">
       <c r="B21" s="80" t="inlineStr">
@@ -3477,16 +3489,16 @@
       <c r="Q31" s="76" t="n"/>
     </row>
     <row r="32" ht="15.75" customFormat="1" customHeight="1" s="79" thickBot="1">
-      <c r="B32" s="32" t="inlineStr">
+      <c r="B32" s="117" t="inlineStr">
         <is>
           <t>February</t>
         </is>
       </c>
-      <c r="C32" s="32" t="n"/>
-      <c r="D32" s="103" t="n">
+      <c r="C32" s="117" t="n"/>
+      <c r="D32" s="118" t="n">
         <v>700</v>
       </c>
-      <c r="E32" s="104">
+      <c r="E32" s="119">
         <f>D32*0.85</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Backwrite: auto-populate agency fields from existing order + fix notes spacing
- read_existing_order_fields now returns agency_flag (Agency/Direct) and
  agency_fee (integer %) by searching for the Agency Discount row in the SC sheet
- handleExistingFile JS populates billing_type, agency_flag, agency_fee and
  calls toggleAgencyFee() when loading an existing order
- Fix notes double-spacing: strip \r\n → \n before writing to Excel
- template.xlsx: Run Sheet estimate placeholder updated to <estimate_run>

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/backwrite/template.xlsx
+++ b/src/backwrite/template.xlsx
@@ -3874,7 +3874,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P2" s="108" t="inlineStr">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P3" s="108" t="inlineStr">
@@ -4142,7 +4142,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P4" s="108" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P5" s="108" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P6" s="108" t="inlineStr">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P7" s="108" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P8" s="108" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P9" s="108" t="inlineStr">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P10" s="108" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P11" s="108" t="inlineStr">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P12" s="108" t="inlineStr">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>&lt;estimate&gt;</t>
+          <t>&lt;estimate_run&gt;</t>
         </is>
       </c>
       <c r="P13" s="108" t="inlineStr">

</xml_diff>

<commit_message>
backwrite: fix gross-up on run sheet; use formulas for spot value and station net
- Move gross-up pass out of EtereBridge-specific block so it applies to
  all run rows regardless of path (EtereBridge or fallback). Previously
  the fallback path never grossed up run rows, causing the run sheet to
  show net rates while the Sales Confirmation tab showed grossed-up rates.

- Replace <spot_value> and <station_net> run sheet template placeholders
  with Excel formulas (=P{row} and =P{row}-T{row}). Gross Rate and Broker
  Fees remain server-written since they require external inputs (grossed-up
  rate and variable commission including zero cases).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/backwrite/template.xlsx
+++ b/src/backwrite/template.xlsx
@@ -3882,10 +3882,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R2" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R2" s="108">
+        <f>P2</f>
+        <v/>
       </c>
       <c r="S2" s="51" t="inlineStr">
         <is>
@@ -3902,10 +3901,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V2" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V2" s="108">
+        <f>P2-T2</f>
+        <v/>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -4016,10 +4014,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R3" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R3" s="108">
+        <f>P3</f>
+        <v/>
       </c>
       <c r="S3" s="51" t="inlineStr">
         <is>
@@ -4036,10 +4033,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V3" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V3" s="108">
+        <f>P3-T3</f>
+        <v/>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -4150,10 +4146,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R4" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R4" s="108">
+        <f>P4</f>
+        <v/>
       </c>
       <c r="S4" s="51" t="inlineStr">
         <is>
@@ -4170,10 +4165,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V4" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V4" s="108">
+        <f>P4-T4</f>
+        <v/>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -4284,10 +4278,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R5" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R5" s="108">
+        <f>P5</f>
+        <v/>
       </c>
       <c r="S5" s="51" t="inlineStr">
         <is>
@@ -4304,10 +4297,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V5" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V5" s="108">
+        <f>P5-T5</f>
+        <v/>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -4418,10 +4410,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R6" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R6" s="108">
+        <f>P6</f>
+        <v/>
       </c>
       <c r="S6" s="51" t="inlineStr">
         <is>
@@ -4438,10 +4429,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V6" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V6" s="108">
+        <f>P6-T6</f>
+        <v/>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -4552,10 +4542,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R7" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R7" s="108">
+        <f>P7</f>
+        <v/>
       </c>
       <c r="S7" s="51" t="inlineStr">
         <is>
@@ -4572,10 +4561,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V7" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V7" s="108">
+        <f>P7-T7</f>
+        <v/>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -4686,10 +4674,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R8" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R8" s="108">
+        <f>P8</f>
+        <v/>
       </c>
       <c r="S8" s="51" t="inlineStr">
         <is>
@@ -4706,10 +4693,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V8" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V8" s="108">
+        <f>P8-T8</f>
+        <v/>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -4820,10 +4806,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R9" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R9" s="108">
+        <f>P9</f>
+        <v/>
       </c>
       <c r="S9" s="51" t="inlineStr">
         <is>
@@ -4840,10 +4825,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V9" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V9" s="108">
+        <f>P9-T9</f>
+        <v/>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -4954,10 +4938,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R10" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R10" s="108">
+        <f>P10</f>
+        <v/>
       </c>
       <c r="S10" s="51" t="inlineStr">
         <is>
@@ -4974,10 +4957,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V10" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V10" s="108">
+        <f>P10-T10</f>
+        <v/>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -5088,10 +5070,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R11" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R11" s="108">
+        <f>P11</f>
+        <v/>
       </c>
       <c r="S11" s="51" t="inlineStr">
         <is>
@@ -5108,10 +5089,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V11" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V11" s="108">
+        <f>P11-T11</f>
+        <v/>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -5222,10 +5202,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R12" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R12" s="108">
+        <f>P12</f>
+        <v/>
       </c>
       <c r="S12" s="51" t="inlineStr">
         <is>
@@ -5242,10 +5221,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V12" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V12" s="108">
+        <f>P12-T12</f>
+        <v/>
       </c>
       <c r="W12" t="inlineStr">
         <is>
@@ -5356,10 +5334,9 @@
           <t>&lt;gross_rate&gt;</t>
         </is>
       </c>
-      <c r="R13" s="108" t="inlineStr">
-        <is>
-          <t>&lt;spot_value&gt;</t>
-        </is>
+      <c r="R13" s="108">
+        <f>P13</f>
+        <v/>
       </c>
       <c r="S13" s="51" t="inlineStr">
         <is>
@@ -5376,10 +5353,9 @@
           <t>&lt;priority&gt;</t>
         </is>
       </c>
-      <c r="V13" s="108" t="inlineStr">
-        <is>
-          <t>&lt;station_net&gt;</t>
-        </is>
+      <c r="V13" s="108">
+        <f>P13-T13</f>
+        <v/>
       </c>
       <c r="W13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(backwrite): template saved with cursor at A1 on every tab
</commit_message>
<xml_diff>
--- a/src/backwrite/template.xlsx
+++ b/src/backwrite/template.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\scrib\dev\ctv-orderentry\src\backwrite\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usrjp\windev\ctv-orderentry\src\backwrite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_F120129DD0788EE565B47F81C7C59CF1AF3AB3DA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sales Confirmation" sheetId="1" r:id="rId1"/>
@@ -20,23 +19,10 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Run Sheet'!$A$1:$AC$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -391,7 +377,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="7">
     <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
@@ -1105,35 +1091,17 @@
   </cellStyleXfs>
   <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="24" borderId="11" xfId="78" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="24" borderId="11" xfId="78" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="24" borderId="11" xfId="78" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="21" fontId="4" fillId="24" borderId="11" xfId="78" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="24" borderId="11" xfId="55" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1142,24 +1110,11 @@
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="56" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1173,20 +1128,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="55" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="55" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1196,9 +1142,6 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="4" fillId="24" borderId="11" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1208,29 +1151,72 @@
     <xf numFmtId="46" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="56" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="24" borderId="11" xfId="78" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="24" borderId="11" xfId="55" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="55" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="56" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="55" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="7" fontId="6" fillId="0" borderId="0" xfId="56" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="56" applyNumberFormat="1"/>
     <xf numFmtId="7" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1296,95 +1282,95 @@
     </xf>
   </cellXfs>
   <cellStyles count="89">
-    <cellStyle name="20% - Accent1 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="20% - Accent1 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="20% - Accent2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="20% - Accent2 3" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="20% - Accent3 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="20% - Accent3 3" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="20% - Accent4 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="20% - Accent4 3" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="20% - Accent5 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="20% - Accent5 3" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="20% - Accent6 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="20% - Accent6 3" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="40% - Accent1 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="40% - Accent1 3" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="40% - Accent2 2" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="40% - Accent2 3" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="40% - Accent3 2" xfId="17" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
-    <cellStyle name="40% - Accent3 3" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="40% - Accent4 2" xfId="19" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
-    <cellStyle name="40% - Accent4 3" xfId="20" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
-    <cellStyle name="40% - Accent5 2" xfId="21" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
-    <cellStyle name="40% - Accent5 3" xfId="22" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
-    <cellStyle name="40% - Accent6 2" xfId="23" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
-    <cellStyle name="40% - Accent6 3" xfId="24" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
-    <cellStyle name="60% - Accent1 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
-    <cellStyle name="60% - Accent1 3" xfId="26" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
-    <cellStyle name="60% - Accent2 2" xfId="27" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
-    <cellStyle name="60% - Accent2 3" xfId="28" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
-    <cellStyle name="60% - Accent3 2" xfId="29" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
-    <cellStyle name="60% - Accent3 3" xfId="30" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
-    <cellStyle name="60% - Accent4 2" xfId="31" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
-    <cellStyle name="60% - Accent4 3" xfId="32" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
-    <cellStyle name="60% - Accent5 2" xfId="33" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
-    <cellStyle name="60% - Accent5 3" xfId="34" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
-    <cellStyle name="60% - Accent6 2" xfId="35" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
-    <cellStyle name="60% - Accent6 3" xfId="36" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
-    <cellStyle name="Accent1 2" xfId="37" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
-    <cellStyle name="Accent1 3" xfId="38" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
-    <cellStyle name="Accent2 2" xfId="39" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
-    <cellStyle name="Accent2 3" xfId="40" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
-    <cellStyle name="Accent3 2" xfId="41" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
-    <cellStyle name="Accent3 3" xfId="42" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
-    <cellStyle name="Accent4 2" xfId="43" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
-    <cellStyle name="Accent4 3" xfId="44" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
-    <cellStyle name="Accent5 2" xfId="45" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
-    <cellStyle name="Accent5 3" xfId="46" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
-    <cellStyle name="Accent6 2" xfId="47" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
-    <cellStyle name="Accent6 3" xfId="48" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
-    <cellStyle name="Bad 2" xfId="49" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
-    <cellStyle name="Bad 3" xfId="50" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
-    <cellStyle name="Calculation 2" xfId="51" xr:uid="{00000000-0005-0000-0000-000033000000}"/>
-    <cellStyle name="Calculation 3" xfId="52" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
-    <cellStyle name="Check Cell 2" xfId="53" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
-    <cellStyle name="Check Cell 3" xfId="54" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
+    <cellStyle name="20% - Accent1 2" xfId="1"/>
+    <cellStyle name="20% - Accent1 3" xfId="2"/>
+    <cellStyle name="20% - Accent2 2" xfId="3"/>
+    <cellStyle name="20% - Accent2 3" xfId="4"/>
+    <cellStyle name="20% - Accent3 2" xfId="5"/>
+    <cellStyle name="20% - Accent3 3" xfId="6"/>
+    <cellStyle name="20% - Accent4 2" xfId="7"/>
+    <cellStyle name="20% - Accent4 3" xfId="8"/>
+    <cellStyle name="20% - Accent5 2" xfId="9"/>
+    <cellStyle name="20% - Accent5 3" xfId="10"/>
+    <cellStyle name="20% - Accent6 2" xfId="11"/>
+    <cellStyle name="20% - Accent6 3" xfId="12"/>
+    <cellStyle name="40% - Accent1 2" xfId="13"/>
+    <cellStyle name="40% - Accent1 3" xfId="14"/>
+    <cellStyle name="40% - Accent2 2" xfId="15"/>
+    <cellStyle name="40% - Accent2 3" xfId="16"/>
+    <cellStyle name="40% - Accent3 2" xfId="17"/>
+    <cellStyle name="40% - Accent3 3" xfId="18"/>
+    <cellStyle name="40% - Accent4 2" xfId="19"/>
+    <cellStyle name="40% - Accent4 3" xfId="20"/>
+    <cellStyle name="40% - Accent5 2" xfId="21"/>
+    <cellStyle name="40% - Accent5 3" xfId="22"/>
+    <cellStyle name="40% - Accent6 2" xfId="23"/>
+    <cellStyle name="40% - Accent6 3" xfId="24"/>
+    <cellStyle name="60% - Accent1 2" xfId="25"/>
+    <cellStyle name="60% - Accent1 3" xfId="26"/>
+    <cellStyle name="60% - Accent2 2" xfId="27"/>
+    <cellStyle name="60% - Accent2 3" xfId="28"/>
+    <cellStyle name="60% - Accent3 2" xfId="29"/>
+    <cellStyle name="60% - Accent3 3" xfId="30"/>
+    <cellStyle name="60% - Accent4 2" xfId="31"/>
+    <cellStyle name="60% - Accent4 3" xfId="32"/>
+    <cellStyle name="60% - Accent5 2" xfId="33"/>
+    <cellStyle name="60% - Accent5 3" xfId="34"/>
+    <cellStyle name="60% - Accent6 2" xfId="35"/>
+    <cellStyle name="60% - Accent6 3" xfId="36"/>
+    <cellStyle name="Accent1 2" xfId="37"/>
+    <cellStyle name="Accent1 3" xfId="38"/>
+    <cellStyle name="Accent2 2" xfId="39"/>
+    <cellStyle name="Accent2 3" xfId="40"/>
+    <cellStyle name="Accent3 2" xfId="41"/>
+    <cellStyle name="Accent3 3" xfId="42"/>
+    <cellStyle name="Accent4 2" xfId="43"/>
+    <cellStyle name="Accent4 3" xfId="44"/>
+    <cellStyle name="Accent5 2" xfId="45"/>
+    <cellStyle name="Accent5 3" xfId="46"/>
+    <cellStyle name="Accent6 2" xfId="47"/>
+    <cellStyle name="Accent6 3" xfId="48"/>
+    <cellStyle name="Bad 2" xfId="49"/>
+    <cellStyle name="Bad 3" xfId="50"/>
+    <cellStyle name="Calculation 2" xfId="51"/>
+    <cellStyle name="Calculation 3" xfId="52"/>
+    <cellStyle name="Check Cell 2" xfId="53"/>
+    <cellStyle name="Check Cell 3" xfId="54"/>
     <cellStyle name="Currency" xfId="55" builtinId="4"/>
-    <cellStyle name="Currency 2" xfId="56" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
-    <cellStyle name="Currency 3" xfId="57" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
-    <cellStyle name="Explanatory Text 2" xfId="58" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
-    <cellStyle name="Explanatory Text 3" xfId="59" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
-    <cellStyle name="Good 2" xfId="60" xr:uid="{00000000-0005-0000-0000-00003C000000}"/>
-    <cellStyle name="Good 3" xfId="61" xr:uid="{00000000-0005-0000-0000-00003D000000}"/>
-    <cellStyle name="Heading 1 2" xfId="62" xr:uid="{00000000-0005-0000-0000-00003E000000}"/>
-    <cellStyle name="Heading 1 3" xfId="63" xr:uid="{00000000-0005-0000-0000-00003F000000}"/>
-    <cellStyle name="Heading 2 2" xfId="64" xr:uid="{00000000-0005-0000-0000-000040000000}"/>
-    <cellStyle name="Heading 2 3" xfId="65" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
-    <cellStyle name="Heading 3 2" xfId="66" xr:uid="{00000000-0005-0000-0000-000042000000}"/>
-    <cellStyle name="Heading 3 3" xfId="67" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
-    <cellStyle name="Heading 4 2" xfId="68" xr:uid="{00000000-0005-0000-0000-000044000000}"/>
-    <cellStyle name="Heading 4 3" xfId="69" xr:uid="{00000000-0005-0000-0000-000045000000}"/>
+    <cellStyle name="Currency 2" xfId="56"/>
+    <cellStyle name="Currency 3" xfId="57"/>
+    <cellStyle name="Explanatory Text 2" xfId="58"/>
+    <cellStyle name="Explanatory Text 3" xfId="59"/>
+    <cellStyle name="Good 2" xfId="60"/>
+    <cellStyle name="Good 3" xfId="61"/>
+    <cellStyle name="Heading 1 2" xfId="62"/>
+    <cellStyle name="Heading 1 3" xfId="63"/>
+    <cellStyle name="Heading 2 2" xfId="64"/>
+    <cellStyle name="Heading 2 3" xfId="65"/>
+    <cellStyle name="Heading 3 2" xfId="66"/>
+    <cellStyle name="Heading 3 3" xfId="67"/>
+    <cellStyle name="Heading 4 2" xfId="68"/>
+    <cellStyle name="Heading 4 3" xfId="69"/>
     <cellStyle name="Hyperlink" xfId="70" builtinId="8"/>
-    <cellStyle name="Input 2" xfId="71" xr:uid="{00000000-0005-0000-0000-000047000000}"/>
-    <cellStyle name="Input 3" xfId="72" xr:uid="{00000000-0005-0000-0000-000048000000}"/>
-    <cellStyle name="Linked Cell 2" xfId="73" xr:uid="{00000000-0005-0000-0000-000049000000}"/>
-    <cellStyle name="Linked Cell 3" xfId="74" xr:uid="{00000000-0005-0000-0000-00004A000000}"/>
-    <cellStyle name="Neutral 2" xfId="75" xr:uid="{00000000-0005-0000-0000-00004B000000}"/>
-    <cellStyle name="Neutral 3" xfId="76" xr:uid="{00000000-0005-0000-0000-00004C000000}"/>
+    <cellStyle name="Input 2" xfId="71"/>
+    <cellStyle name="Input 3" xfId="72"/>
+    <cellStyle name="Linked Cell 2" xfId="73"/>
+    <cellStyle name="Linked Cell 3" xfId="74"/>
+    <cellStyle name="Neutral 2" xfId="75"/>
+    <cellStyle name="Neutral 3" xfId="76"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="77" xr:uid="{00000000-0005-0000-0000-00004D000000}"/>
-    <cellStyle name="Normal_10 06 03" xfId="78" xr:uid="{00000000-0005-0000-0000-00004E000000}"/>
-    <cellStyle name="Note 2" xfId="79" xr:uid="{00000000-0005-0000-0000-00004F000000}"/>
-    <cellStyle name="Note 3" xfId="80" xr:uid="{00000000-0005-0000-0000-000050000000}"/>
-    <cellStyle name="Output 2" xfId="81" xr:uid="{00000000-0005-0000-0000-000051000000}"/>
-    <cellStyle name="Output 3" xfId="82" xr:uid="{00000000-0005-0000-0000-000052000000}"/>
-    <cellStyle name="Title 2" xfId="83" xr:uid="{00000000-0005-0000-0000-000053000000}"/>
-    <cellStyle name="Title 3" xfId="84" xr:uid="{00000000-0005-0000-0000-000054000000}"/>
-    <cellStyle name="Total 2" xfId="85" xr:uid="{00000000-0005-0000-0000-000055000000}"/>
-    <cellStyle name="Total 3" xfId="86" xr:uid="{00000000-0005-0000-0000-000056000000}"/>
-    <cellStyle name="Warning Text 2" xfId="87" xr:uid="{00000000-0005-0000-0000-000057000000}"/>
-    <cellStyle name="Warning Text 3" xfId="88" xr:uid="{00000000-0005-0000-0000-000058000000}"/>
+    <cellStyle name="Normal 2" xfId="77"/>
+    <cellStyle name="Normal_10 06 03" xfId="78"/>
+    <cellStyle name="Note 2" xfId="79"/>
+    <cellStyle name="Note 3" xfId="80"/>
+    <cellStyle name="Output 2" xfId="81"/>
+    <cellStyle name="Output 3" xfId="82"/>
+    <cellStyle name="Title 2" xfId="83"/>
+    <cellStyle name="Title 3" xfId="84"/>
+    <cellStyle name="Total 2" xfId="85"/>
+    <cellStyle name="Total 3" xfId="86"/>
+    <cellStyle name="Warning Text 2" xfId="87"/>
+    <cellStyle name="Warning Text 3" xfId="88"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1400,7 +1386,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Lee Hudson" refreshedDate="46127.677987731477" createdVersion="4" refreshedVersion="8" minRefreshableVersion="3" recordCount="25" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="Lee Hudson" refreshedDate="46127.677987731477" createdVersion="4" refreshedVersion="8" minRefreshableVersion="3" recordCount="25">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:AC1048576" sheet="Run Sheet"/>
   </cacheSource>
@@ -2335,7 +2321,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="4" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:C6" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="29">
     <pivotField showAll="0"/>
@@ -2454,11 +2440,6 @@
     <dataField name="Sum of Station Net" fld="21" baseField="18" baseItem="6" numFmtId="167"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
 </pivotTableDefinition>
 </file>
 
@@ -2748,50 +2729,50 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet40">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AJ36"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" style="21" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="11" style="22" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="22" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" style="22" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" style="22" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.28515625" style="21" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="22" customWidth="1"/>
-    <col min="10" max="10" width="5.85546875" style="22" customWidth="1"/>
-    <col min="11" max="11" width="6.42578125" style="22" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="10" style="22" customWidth="1"/>
-    <col min="13" max="13" width="10" style="22" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="11.5703125" style="22" customWidth="1"/>
-    <col min="16" max="16" width="14" style="22" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" style="22" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.85546875" style="21" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="6.7109375" style="21" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="10.5703125" style="21" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="26.5703125" style="21" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="10.140625" style="21" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="11" style="21" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="11.7109375" style="21" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="10.140625" style="21" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="7.140625" style="21" hidden="1" customWidth="1"/>
-    <col min="27" max="28" width="8.42578125" style="21" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="6.42578125" style="21" hidden="1" customWidth="1"/>
-    <col min="30" max="36" width="13" style="21" hidden="1" customWidth="1"/>
-    <col min="37" max="37" width="149.140625" style="21" hidden="1" customWidth="1"/>
-    <col min="38" max="16384" width="149.140625" style="21" hidden="1"/>
+    <col min="1" max="1" width="23.28515625" style="10" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="11" style="11" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="11" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="11" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.28515625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="11" customWidth="1"/>
+    <col min="10" max="10" width="5.85546875" style="11" customWidth="1"/>
+    <col min="11" max="11" width="6.42578125" style="11" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="10" style="11" customWidth="1"/>
+    <col min="13" max="13" width="10" style="11" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="11.5703125" style="11" customWidth="1"/>
+    <col min="16" max="16" width="14" style="11" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" style="11" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" style="10" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="6.7109375" style="10" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="10.5703125" style="10" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="26.5703125" style="10" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" style="10" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="11" style="10" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="11.7109375" style="10" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="10.140625" style="10" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="7.140625" style="10" hidden="1" customWidth="1"/>
+    <col min="27" max="28" width="8.42578125" style="10" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="6.42578125" style="10" hidden="1" customWidth="1"/>
+    <col min="30" max="36" width="13" style="10" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="149.140625" style="10" hidden="1" customWidth="1"/>
+    <col min="38" max="16384" width="149.140625" style="10" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="1"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
       <c r="F1" s="73" t="s">
         <v>0</v>
       </c>
@@ -2801,45 +2782,45 @@
       <c r="J1" s="69"/>
       <c r="K1" s="69"/>
       <c r="L1" s="69"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
     </row>
     <row r="2" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="3"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="65" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="64"/>
       <c r="F3" s="64"/>
       <c r="G3" s="64"/>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
       <c r="L3" s="68" t="s">
         <v>4</v>
       </c>
@@ -2850,17 +2831,17 @@
       <c r="Q3" s="69"/>
     </row>
     <row r="4" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="1"/>
       <c r="D4" s="82" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="67"/>
       <c r="F4" s="67"/>
       <c r="G4" s="67"/>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="38" t="s">
         <v>7</v>
       </c>
       <c r="L4" s="68" t="s">
@@ -2873,21 +2854,21 @@
       <c r="Q4" s="69"/>
     </row>
     <row r="5" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="1"/>
+      <c r="D5" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="I5" s="3" t="s">
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="I5" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
       <c r="L5" s="68" t="s">
         <v>12</v>
       </c>
@@ -2898,23 +2879,23 @@
       <c r="Q5" s="69"/>
     </row>
     <row r="6" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="1"/>
-      <c r="C6" s="2"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="1"/>
       <c r="D6" s="65" t="s">
         <v>13</v>
       </c>
       <c r="E6" s="64"/>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
       <c r="L6" s="68" t="s">
         <v>17</v>
       </c>
@@ -2925,29 +2906,29 @@
       <c r="Q6" s="69"/>
     </row>
     <row r="7" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
     </row>
     <row r="8" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="1"/>
       <c r="D8" s="63" t="s">
         <v>19</v>
       </c>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
       <c r="L8" s="70" t="s">
         <v>21</v>
       </c>
@@ -2958,63 +2939,63 @@
       <c r="Q8" s="69"/>
     </row>
     <row r="9" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="1"/>
       <c r="D9" s="63" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="64"/>
       <c r="F9" s="64"/>
       <c r="G9" s="64"/>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="4" t="s">
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="31"/>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="31"/>
     </row>
     <row r="10" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="2"/>
+      <c r="C10" s="1"/>
       <c r="D10" s="66" t="s">
         <v>27</v>
       </c>
       <c r="E10" s="67"/>
       <c r="F10" s="67"/>
       <c r="G10" s="67"/>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="L10" s="4">
+      <c r="L10" s="31">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="1"/>
       <c r="D11" s="66" t="s">
         <v>29</v>
       </c>
       <c r="E11" s="67"/>
       <c r="F11" s="67"/>
       <c r="G11" s="67"/>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="J11" s="2"/>
+      <c r="J11" s="1"/>
       <c r="K11" s="68" t="s">
         <v>31</v>
       </c>
@@ -3026,286 +3007,286 @@
       <c r="Q11" s="69"/>
     </row>
     <row r="12" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="1"/>
       <c r="D12" s="66" t="s">
         <v>32</v>
       </c>
       <c r="E12" s="67"/>
       <c r="F12" s="67"/>
       <c r="G12" s="67"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="31"/>
+      <c r="N12" s="31"/>
+      <c r="O12" s="31"/>
+      <c r="P12" s="31"/>
+      <c r="Q12" s="31"/>
     </row>
     <row r="13" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="1"/>
       <c r="D13" s="66" t="s">
         <v>33</v>
       </c>
       <c r="E13" s="67"/>
       <c r="F13" s="67"/>
       <c r="G13" s="67"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="4"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="31"/>
+      <c r="O13" s="31"/>
+      <c r="P13" s="31"/>
+      <c r="Q13" s="31"/>
     </row>
     <row r="14" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="1"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="24"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-    </row>
-    <row r="15" spans="2:22" s="5" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="6" t="s">
+      <c r="B14" s="30"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="13"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="31"/>
+      <c r="N14" s="31"/>
+      <c r="O14" s="31"/>
+      <c r="P14" s="31"/>
+      <c r="Q14" s="31"/>
+    </row>
+    <row r="15" spans="2:22" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="5" t="s">
+      <c r="C15" s="3"/>
+      <c r="D15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="L15" s="5" t="s">
+      <c r="L15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="N15" s="5" t="s">
+      <c r="N15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="O15" s="9" t="s">
+      <c r="O15" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="P15" s="5" t="s">
+      <c r="P15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-      <c r="T15" s="9"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-    </row>
-    <row r="16" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="37">
+      <c r="R15" s="42"/>
+      <c r="S15" s="42"/>
+      <c r="T15" s="42"/>
+      <c r="U15" s="42"/>
+      <c r="V15" s="42"/>
+    </row>
+    <row r="16" spans="2:22" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="33">
         <v>1</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12" t="s">
+      <c r="C16" s="5"/>
+      <c r="D16" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="37" t="s">
+      <c r="F16" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="G16" s="13" t="s">
+      <c r="G16" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="I16" s="37">
+      <c r="I16" s="33">
         <v>1</v>
       </c>
-      <c r="J16" s="37" t="s">
+      <c r="J16" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="L16" s="37" t="e">
+      <c r="L16" s="33" t="e">
         <f>F16*I16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N16" s="37" t="s">
+      <c r="N16" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="O16" s="26" t="s">
+      <c r="O16" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="P16" s="26" t="e">
+      <c r="P16" s="44" t="e">
         <f>L16*O16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R16" s="14"/>
-      <c r="T16" s="14"/>
-      <c r="U16" s="14"/>
-      <c r="V16" s="14"/>
-    </row>
-    <row r="17" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="37">
+      <c r="R16" s="45"/>
+      <c r="T16" s="45"/>
+      <c r="U16" s="45"/>
+      <c r="V16" s="45"/>
+    </row>
+    <row r="17" spans="2:22" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="33">
         <v>2</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="12" t="s">
+      <c r="C17" s="5"/>
+      <c r="D17" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F17" s="37" t="s">
+      <c r="F17" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="G17" s="13" t="s">
+      <c r="G17" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="I17" s="37">
+      <c r="I17" s="33">
         <v>1</v>
       </c>
-      <c r="J17" s="37" t="s">
+      <c r="J17" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="L17" s="37" t="e">
+      <c r="L17" s="33" t="e">
         <f>F17*I17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N17" s="37" t="s">
+      <c r="N17" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="O17" s="26" t="s">
+      <c r="O17" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="P17" s="26" t="e">
+      <c r="P17" s="44" t="e">
         <f>L17*O17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R17" s="14"/>
-      <c r="T17" s="14"/>
-      <c r="U17" s="14"/>
-      <c r="V17" s="14"/>
-    </row>
-    <row r="18" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="37">
+      <c r="R17" s="45"/>
+      <c r="T17" s="45"/>
+      <c r="U17" s="45"/>
+      <c r="V17" s="45"/>
+    </row>
+    <row r="18" spans="2:22" s="32" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="33">
         <v>3</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12" t="s">
+      <c r="C18" s="5"/>
+      <c r="D18" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F18" s="37" t="s">
+      <c r="F18" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="G18" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="I18" s="37">
+      <c r="I18" s="33">
         <v>1</v>
       </c>
-      <c r="J18" s="37" t="s">
+      <c r="J18" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="L18" s="37" t="e">
+      <c r="L18" s="33" t="e">
         <f>F18*I18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N18" s="37" t="s">
+      <c r="N18" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="O18" s="26" t="s">
+      <c r="O18" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="P18" s="26" t="e">
+      <c r="P18" s="44" t="e">
         <f>L18*O18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R18" s="14"/>
-      <c r="T18" s="14"/>
-      <c r="U18" s="14"/>
-      <c r="V18" s="14"/>
-    </row>
-    <row r="19" spans="2:22" s="10" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="37">
+      <c r="R18" s="45"/>
+      <c r="T18" s="45"/>
+      <c r="U18" s="45"/>
+      <c r="V18" s="45"/>
+    </row>
+    <row r="19" spans="2:22" s="32" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="33">
         <v>4</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12" t="s">
+      <c r="C19" s="5"/>
+      <c r="D19" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F19" s="37" t="s">
+      <c r="F19" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="G19" s="13" t="s">
+      <c r="G19" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="I19" s="37">
+      <c r="I19" s="33">
         <v>1</v>
       </c>
-      <c r="J19" s="37" t="s">
+      <c r="J19" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="L19" s="37" t="e">
+      <c r="L19" s="33" t="e">
         <f>F19*I19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N19" s="37" t="s">
+      <c r="N19" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="O19" s="26" t="s">
+      <c r="O19" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="P19" s="26" t="e">
+      <c r="P19" s="44" t="e">
         <f>L19*O19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="R19" s="14"/>
-      <c r="T19" s="14"/>
-      <c r="U19" s="14"/>
-      <c r="V19" s="14"/>
-    </row>
-    <row r="20" spans="2:22" s="15" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R19" s="45"/>
+      <c r="T19" s="45"/>
+      <c r="U19" s="45"/>
+      <c r="V19" s="45"/>
+    </row>
+    <row r="20" spans="2:22" s="7" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B20" s="53"/>
       <c r="C20" s="53"/>
       <c r="D20" s="54"/>
@@ -3332,7 +3313,7 @@
       </c>
       <c r="Q20" s="59"/>
     </row>
-    <row r="21" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="73" t="s">
         <v>57</v>
       </c>
@@ -3341,25 +3322,25 @@
       <c r="E21" s="72"/>
       <c r="F21" s="72"/>
       <c r="G21" s="72"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="48" t="s">
+      <c r="H21" s="34"/>
+      <c r="I21" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="J21" s="49"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="51">
+      <c r="J21" s="35"/>
+      <c r="K21" s="35"/>
+      <c r="L21" s="40">
         <v>0.15</v>
       </c>
-      <c r="M21" s="49"/>
-      <c r="N21" s="49"/>
-      <c r="O21" s="50"/>
-      <c r="P21" s="52" t="e">
+      <c r="M21" s="35"/>
+      <c r="N21" s="35"/>
+      <c r="O21" s="37"/>
+      <c r="P21" s="46" t="e">
         <f>-1*(L21*P20)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Q21" s="17"/>
-    </row>
-    <row r="22" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q21" s="36"/>
+    </row>
+    <row r="22" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="75" t="s">
         <v>59</v>
       </c>
@@ -3368,181 +3349,181 @@
       <c r="E22" s="76"/>
       <c r="F22" s="76"/>
       <c r="G22" s="77"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3" t="s">
+      <c r="H22" s="38"/>
+      <c r="I22" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="19"/>
-      <c r="O22" s="19"/>
-      <c r="P22" s="20" t="s">
+      <c r="J22" s="36"/>
+      <c r="K22" s="36"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="Q22" s="17"/>
-    </row>
-    <row r="23" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="Q22" s="36"/>
+    </row>
+    <row r="23" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B23" s="78"/>
       <c r="C23" s="72"/>
       <c r="D23" s="72"/>
       <c r="E23" s="72"/>
       <c r="F23" s="72"/>
       <c r="G23" s="79"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="17"/>
-      <c r="O23" s="17"/>
-      <c r="P23" s="17"/>
-      <c r="Q23" s="17"/>
-    </row>
-    <row r="24" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
+      <c r="K23" s="36"/>
+      <c r="L23" s="36"/>
+      <c r="M23" s="36"/>
+      <c r="N23" s="36"/>
+      <c r="O23" s="36"/>
+      <c r="P23" s="36"/>
+      <c r="Q23" s="36"/>
+    </row>
+    <row r="24" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="78"/>
       <c r="C24" s="72"/>
       <c r="D24" s="72"/>
       <c r="E24" s="72"/>
       <c r="F24" s="72"/>
       <c r="G24" s="79"/>
-      <c r="I24" s="3" t="s">
+      <c r="I24" s="38" t="s">
         <v>62</v>
       </c>
-      <c r="J24" s="17"/>
-      <c r="K24" s="17"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="25"/>
-      <c r="N24" s="25"/>
-      <c r="O24" s="25"/>
-      <c r="P24" s="25"/>
-      <c r="Q24" s="17"/>
-    </row>
-    <row r="25" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J24" s="36"/>
+      <c r="K24" s="36"/>
+      <c r="L24" s="14"/>
+      <c r="M24" s="14"/>
+      <c r="N24" s="14"/>
+      <c r="O24" s="14"/>
+      <c r="P24" s="14"/>
+      <c r="Q24" s="36"/>
+    </row>
+    <row r="25" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="78"/>
       <c r="C25" s="72"/>
       <c r="D25" s="72"/>
       <c r="E25" s="72"/>
       <c r="F25" s="72"/>
       <c r="G25" s="79"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="17"/>
-      <c r="M25" s="17"/>
-      <c r="N25" s="17"/>
-      <c r="O25" s="17"/>
-      <c r="P25" s="17"/>
-      <c r="Q25" s="17"/>
-    </row>
-    <row r="26" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I25" s="38"/>
+      <c r="J25" s="36"/>
+      <c r="K25" s="36"/>
+      <c r="L25" s="36"/>
+      <c r="M25" s="36"/>
+      <c r="N25" s="36"/>
+      <c r="O25" s="36"/>
+      <c r="P25" s="36"/>
+      <c r="Q25" s="36"/>
+    </row>
+    <row r="26" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="78"/>
       <c r="C26" s="72"/>
       <c r="D26" s="72"/>
       <c r="E26" s="72"/>
       <c r="F26" s="72"/>
       <c r="G26" s="79"/>
-      <c r="I26" s="3" t="s">
+      <c r="I26" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="25"/>
-      <c r="M26" s="25"/>
-      <c r="N26" s="25"/>
-      <c r="O26" s="25"/>
-      <c r="P26" s="25"/>
-      <c r="Q26" s="17"/>
-    </row>
-    <row r="27" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J26" s="36"/>
+      <c r="K26" s="36"/>
+      <c r="L26" s="14"/>
+      <c r="M26" s="14"/>
+      <c r="N26" s="14"/>
+      <c r="O26" s="14"/>
+      <c r="P26" s="14"/>
+      <c r="Q26" s="36"/>
+    </row>
+    <row r="27" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="80"/>
       <c r="C27" s="64"/>
       <c r="D27" s="64"/>
       <c r="E27" s="64"/>
       <c r="F27" s="64"/>
       <c r="G27" s="81"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="23"/>
-      <c r="N27" s="23"/>
-      <c r="O27" s="23"/>
-      <c r="P27" s="23"/>
-      <c r="Q27" s="17"/>
-    </row>
-    <row r="28" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23"/>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="17"/>
-    </row>
-    <row r="29" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12"/>
+      <c r="O27" s="12"/>
+      <c r="P27" s="12"/>
+      <c r="Q27" s="36"/>
+    </row>
+    <row r="28" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I28" s="12"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="12"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12"/>
+      <c r="O28" s="12"/>
+      <c r="P28" s="12"/>
+      <c r="Q28" s="36"/>
+    </row>
+    <row r="29" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="71" t="s">
         <v>64</v>
       </c>
       <c r="C29" s="72"/>
       <c r="D29" s="72"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="23"/>
-      <c r="K29" s="23"/>
-      <c r="L29" s="23"/>
-      <c r="M29" s="23"/>
-      <c r="N29" s="23"/>
-      <c r="O29" s="23"/>
-      <c r="P29" s="23"/>
-      <c r="Q29" s="17"/>
-    </row>
-    <row r="30" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="23"/>
-      <c r="K30" s="23"/>
-      <c r="L30" s="23"/>
-      <c r="M30" s="23"/>
-      <c r="N30" s="23"/>
-      <c r="O30" s="23"/>
-      <c r="P30" s="23"/>
-      <c r="Q30" s="17"/>
-    </row>
-    <row r="31" spans="2:22" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="1" t="s">
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="12"/>
+      <c r="O29" s="12"/>
+      <c r="P29" s="12"/>
+      <c r="Q29" s="36"/>
+    </row>
+    <row r="30" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="30"/>
+      <c r="C30" s="30"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="12"/>
+      <c r="M30" s="12"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="12"/>
+      <c r="P30" s="12"/>
+      <c r="Q30" s="36"/>
+    </row>
+    <row r="31" spans="2:22" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1" t="s">
+      <c r="C31" s="30"/>
+      <c r="D31" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E31" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
-      <c r="N31" s="23"/>
-      <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
-      <c r="Q31" s="17"/>
-    </row>
-    <row r="32" spans="2:22" s="16" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F31" s="30"/>
+      <c r="G31" s="30"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12"/>
+      <c r="O31" s="12"/>
+      <c r="P31" s="12"/>
+      <c r="Q31" s="36"/>
+    </row>
+    <row r="32" spans="2:22" s="39" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="60" t="s">
         <v>68</v>
       </c>
@@ -3554,91 +3535,91 @@
         <f>D32*0.85</f>
         <v>595</v>
       </c>
-      <c r="I32" s="23"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="23"/>
-      <c r="L32" s="23"/>
-      <c r="M32" s="23"/>
-      <c r="N32" s="23"/>
-      <c r="O32" s="23"/>
-      <c r="P32" s="23"/>
-      <c r="Q32" s="17"/>
-    </row>
-    <row r="33" spans="2:17" s="16" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="30" t="s">
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="12"/>
+      <c r="L32" s="12"/>
+      <c r="M32" s="12"/>
+      <c r="N32" s="12"/>
+      <c r="O32" s="12"/>
+      <c r="P32" s="12"/>
+      <c r="Q32" s="36"/>
+    </row>
+    <row r="33" spans="2:17" s="39" customFormat="1" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="17"/>
-      <c r="D33" s="29">
+      <c r="C33" s="36"/>
+      <c r="D33" s="48">
         <f>SUM(D32:D32)</f>
         <v>700</v>
       </c>
-      <c r="E33" s="31">
+      <c r="E33" s="49">
         <f>SUM(E32:E32)</f>
         <v>595</v>
       </c>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="17"/>
-      <c r="M33" s="17"/>
-      <c r="N33" s="17"/>
-      <c r="O33" s="17"/>
-      <c r="P33" s="17"/>
-      <c r="Q33" s="17"/>
-    </row>
-    <row r="34" spans="2:17" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="17"/>
-      <c r="K34" s="17"/>
-      <c r="L34" s="17"/>
-      <c r="M34" s="17"/>
-      <c r="N34" s="17"/>
-      <c r="O34" s="17"/>
-      <c r="P34" s="17"/>
-      <c r="Q34" s="17"/>
-    </row>
-    <row r="35" spans="2:17" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="17"/>
-      <c r="K35" s="17"/>
-      <c r="L35" s="17"/>
-      <c r="M35" s="17"/>
-      <c r="N35" s="17"/>
-      <c r="O35" s="17"/>
-      <c r="P35" s="17"/>
-      <c r="Q35" s="17"/>
-    </row>
-    <row r="36" spans="2:17" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
-      <c r="G36" s="17"/>
-      <c r="I36" s="17"/>
-      <c r="J36" s="17"/>
-      <c r="K36" s="17"/>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-      <c r="N36" s="17"/>
-      <c r="O36" s="17"/>
-      <c r="P36" s="17"/>
-      <c r="Q36" s="17"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="36"/>
+      <c r="I33" s="36"/>
+      <c r="J33" s="36"/>
+      <c r="K33" s="36"/>
+      <c r="L33" s="36"/>
+      <c r="M33" s="36"/>
+      <c r="N33" s="36"/>
+      <c r="O33" s="36"/>
+      <c r="P33" s="36"/>
+      <c r="Q33" s="36"/>
+    </row>
+    <row r="34" spans="2:17" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="36"/>
+      <c r="C34" s="36"/>
+      <c r="D34" s="36"/>
+      <c r="E34" s="36"/>
+      <c r="F34" s="36"/>
+      <c r="G34" s="36"/>
+      <c r="I34" s="36"/>
+      <c r="J34" s="36"/>
+      <c r="K34" s="36"/>
+      <c r="L34" s="36"/>
+      <c r="M34" s="36"/>
+      <c r="N34" s="36"/>
+      <c r="O34" s="36"/>
+      <c r="P34" s="36"/>
+      <c r="Q34" s="36"/>
+    </row>
+    <row r="35" spans="2:17" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="36"/>
+      <c r="C35" s="36"/>
+      <c r="D35" s="36"/>
+      <c r="E35" s="36"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="36"/>
+      <c r="I35" s="36"/>
+      <c r="J35" s="36"/>
+      <c r="K35" s="36"/>
+      <c r="L35" s="36"/>
+      <c r="M35" s="36"/>
+      <c r="N35" s="36"/>
+      <c r="O35" s="36"/>
+      <c r="P35" s="36"/>
+      <c r="Q35" s="36"/>
+    </row>
+    <row r="36" spans="2:17" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="36"/>
+      <c r="C36" s="36"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="36"/>
+      <c r="I36" s="36"/>
+      <c r="J36" s="36"/>
+      <c r="K36" s="36"/>
+      <c r="L36" s="36"/>
+      <c r="M36" s="36"/>
+      <c r="N36" s="36"/>
+      <c r="O36" s="36"/>
+      <c r="P36" s="36"/>
+      <c r="Q36" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -3663,10 +3644,10 @@
     <mergeCell ref="L8:Q8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D10" r:id="rId1" display="jlee@handlpartners.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="D11" r:id="rId2" display="jlee@handlpartners.com" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="D12" r:id="rId3" display="jlee@handlpartners.com" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="D13" r:id="rId4" display="jlee@handlpartners.com" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D10" r:id="rId1" display="jlee@handlpartners.com"/>
+    <hyperlink ref="D11" r:id="rId2" display="jlee@handlpartners.com"/>
+    <hyperlink ref="D12" r:id="rId3" display="jlee@handlpartners.com"/>
+    <hyperlink ref="D13" r:id="rId4" display="jlee@handlpartners.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="82" fitToHeight="100" orientation="landscape"/>
@@ -3674,7 +3655,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AC25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3695,9 +3676,9 @@
     <col min="16" max="16" width="12.5703125" customWidth="1"/>
     <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="11" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.7109375" style="34" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.7109375" style="20" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="30" style="39" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="30" style="24" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -3708,122 +3689,122 @@
     <col min="29" max="29" width="7.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="5" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:29" s="2" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="41" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="41" t="s">
         <v>74</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="41" t="s">
         <v>76</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="42" t="s">
         <v>82</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="42" t="s">
         <v>84</v>
       </c>
-      <c r="S1" s="33" t="s">
+      <c r="S1" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="U1" s="38" t="s">
+      <c r="U1" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="42" t="s">
         <v>87</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="W1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="X1" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Y1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="Z1" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AA1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AB1" s="38" t="s">
+      <c r="AB1" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AC1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="27" t="str">
+      <c r="C2" s="15" t="str">
         <f t="shared" ref="C2:C13" si="0">B2</f>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D2" s="41" t="s">
+      <c r="D2" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E2" s="42" t="s">
+      <c r="E2" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="42" t="s">
+      <c r="F2" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G2" s="42" t="s">
+      <c r="G2" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H2" t="s">
         <v>98</v>
       </c>
-      <c r="I2" s="43" t="s">
+      <c r="I2" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J2" t="s">
@@ -3841,23 +3822,23 @@
       <c r="O2" t="s">
         <v>102</v>
       </c>
-      <c r="P2" s="44" t="s">
+      <c r="P2" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R2" s="44" t="str">
+      <c r="R2" s="51" t="str">
         <f t="shared" ref="R2:R13" si="1">P2</f>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S2" s="45" t="s">
+      <c r="S2" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T2" s="44" t="s">
+      <c r="T2" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U2" s="46" t="s">
+      <c r="U2" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V2" s="44" t="e">
+      <c r="V2" s="51" t="e">
         <f t="shared" ref="V2:V13" si="2">P2-T2</f>
         <v>#VALUE!</v>
       </c>
@@ -3876,40 +3857,40 @@
       <c r="AA2" t="s">
         <v>109</v>
       </c>
-      <c r="AB2" s="46" t="s">
+      <c r="AB2" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>93</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C3" s="27" t="str">
+      <c r="C3" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F3" s="42" t="s">
+      <c r="F3" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G3" s="42" t="s">
+      <c r="G3" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H3" t="s">
         <v>98</v>
       </c>
-      <c r="I3" s="43" t="s">
+      <c r="I3" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J3" t="s">
@@ -3927,23 +3908,23 @@
       <c r="O3" t="s">
         <v>102</v>
       </c>
-      <c r="P3" s="44" t="s">
+      <c r="P3" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R3" s="44" t="str">
+      <c r="R3" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S3" s="45" t="s">
+      <c r="S3" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T3" s="44" t="s">
+      <c r="T3" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U3" s="46" t="s">
+      <c r="U3" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V3" s="44" t="e">
+      <c r="V3" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -3962,40 +3943,40 @@
       <c r="AA3" t="s">
         <v>109</v>
       </c>
-      <c r="AB3" s="46" t="s">
+      <c r="AB3" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C4" s="27" t="str">
+      <c r="C4" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E4" s="42" t="s">
+      <c r="E4" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G4" s="42" t="s">
+      <c r="G4" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H4" t="s">
         <v>98</v>
       </c>
-      <c r="I4" s="43" t="s">
+      <c r="I4" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J4" t="s">
@@ -4013,23 +3994,23 @@
       <c r="O4" t="s">
         <v>102</v>
       </c>
-      <c r="P4" s="44" t="s">
+      <c r="P4" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R4" s="44" t="str">
+      <c r="R4" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S4" s="45" t="s">
+      <c r="S4" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T4" s="44" t="s">
+      <c r="T4" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U4" s="46" t="s">
+      <c r="U4" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V4" s="44" t="e">
+      <c r="V4" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4048,40 +4029,40 @@
       <c r="AA4" t="s">
         <v>109</v>
       </c>
-      <c r="AB4" s="46" t="s">
+      <c r="AB4" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C5" s="27" t="str">
+      <c r="C5" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E5" s="42" t="s">
+      <c r="E5" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="42" t="s">
+      <c r="F5" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G5" s="42" t="s">
+      <c r="G5" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H5" t="s">
         <v>98</v>
       </c>
-      <c r="I5" s="43" t="s">
+      <c r="I5" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J5" t="s">
@@ -4099,23 +4080,23 @@
       <c r="O5" t="s">
         <v>102</v>
       </c>
-      <c r="P5" s="44" t="s">
+      <c r="P5" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R5" s="44" t="str">
+      <c r="R5" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S5" s="45" t="s">
+      <c r="S5" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T5" s="44" t="s">
+      <c r="T5" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U5" s="46" t="s">
+      <c r="U5" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V5" s="44" t="e">
+      <c r="V5" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4134,40 +4115,40 @@
       <c r="AA5" t="s">
         <v>109</v>
       </c>
-      <c r="AB5" s="46" t="s">
+      <c r="AB5" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C6" s="27" t="str">
+      <c r="C6" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="42" t="s">
+      <c r="F6" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="42" t="s">
+      <c r="G6" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H6" t="s">
         <v>98</v>
       </c>
-      <c r="I6" s="43" t="s">
+      <c r="I6" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J6" t="s">
@@ -4185,23 +4166,23 @@
       <c r="O6" t="s">
         <v>102</v>
       </c>
-      <c r="P6" s="44" t="s">
+      <c r="P6" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R6" s="44" t="str">
+      <c r="R6" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S6" s="45" t="s">
+      <c r="S6" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T6" s="44" t="s">
+      <c r="T6" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U6" s="46" t="s">
+      <c r="U6" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V6" s="44" t="e">
+      <c r="V6" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4220,40 +4201,40 @@
       <c r="AA6" t="s">
         <v>109</v>
       </c>
-      <c r="AB6" s="46" t="s">
+      <c r="AB6" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="27" t="str">
+      <c r="C7" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F7" s="42" t="s">
+      <c r="F7" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G7" s="42" t="s">
+      <c r="G7" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H7" t="s">
         <v>98</v>
       </c>
-      <c r="I7" s="43" t="s">
+      <c r="I7" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J7" t="s">
@@ -4271,23 +4252,23 @@
       <c r="O7" t="s">
         <v>102</v>
       </c>
-      <c r="P7" s="44" t="s">
+      <c r="P7" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R7" s="44" t="str">
+      <c r="R7" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S7" s="45" t="s">
+      <c r="S7" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T7" s="44" t="s">
+      <c r="T7" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U7" s="46" t="s">
+      <c r="U7" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V7" s="44" t="e">
+      <c r="V7" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4306,40 +4287,40 @@
       <c r="AA7" t="s">
         <v>109</v>
       </c>
-      <c r="AB7" s="46" t="s">
+      <c r="AB7" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="27" t="str">
+      <c r="C8" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F8" s="42" t="s">
+      <c r="F8" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G8" s="42" t="s">
+      <c r="G8" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H8" t="s">
         <v>98</v>
       </c>
-      <c r="I8" s="43" t="s">
+      <c r="I8" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J8" t="s">
@@ -4357,23 +4338,23 @@
       <c r="O8" t="s">
         <v>102</v>
       </c>
-      <c r="P8" s="44" t="s">
+      <c r="P8" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R8" s="44" t="str">
+      <c r="R8" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S8" s="45" t="s">
+      <c r="S8" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T8" s="44" t="s">
+      <c r="T8" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U8" s="46" t="s">
+      <c r="U8" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V8" s="44" t="e">
+      <c r="V8" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4392,40 +4373,40 @@
       <c r="AA8" t="s">
         <v>109</v>
       </c>
-      <c r="AB8" s="46" t="s">
+      <c r="AB8" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>93</v>
       </c>
-      <c r="B9" s="40" t="s">
+      <c r="B9" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="27" t="str">
+      <c r="C9" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F9" s="42" t="s">
+      <c r="F9" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G9" s="42" t="s">
+      <c r="G9" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H9" t="s">
         <v>98</v>
       </c>
-      <c r="I9" s="43" t="s">
+      <c r="I9" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J9" t="s">
@@ -4443,23 +4424,23 @@
       <c r="O9" t="s">
         <v>102</v>
       </c>
-      <c r="P9" s="44" t="s">
+      <c r="P9" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R9" s="44" t="str">
+      <c r="R9" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S9" s="45" t="s">
+      <c r="S9" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T9" s="44" t="s">
+      <c r="T9" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U9" s="46" t="s">
+      <c r="U9" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V9" s="44" t="e">
+      <c r="V9" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4478,40 +4459,40 @@
       <c r="AA9" t="s">
         <v>109</v>
       </c>
-      <c r="AB9" s="46" t="s">
+      <c r="AB9" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="27" t="str">
+      <c r="C10" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E10" s="42" t="s">
+      <c r="E10" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F10" s="42" t="s">
+      <c r="F10" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G10" s="42" t="s">
+      <c r="G10" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H10" t="s">
         <v>98</v>
       </c>
-      <c r="I10" s="43" t="s">
+      <c r="I10" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J10" t="s">
@@ -4529,23 +4510,23 @@
       <c r="O10" t="s">
         <v>102</v>
       </c>
-      <c r="P10" s="44" t="s">
+      <c r="P10" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R10" s="44" t="str">
+      <c r="R10" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S10" s="45" t="s">
+      <c r="S10" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T10" s="44" t="s">
+      <c r="T10" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U10" s="46" t="s">
+      <c r="U10" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V10" s="44" t="e">
+      <c r="V10" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4564,40 +4545,40 @@
       <c r="AA10" t="s">
         <v>109</v>
       </c>
-      <c r="AB10" s="46" t="s">
+      <c r="AB10" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="27" t="str">
+      <c r="C11" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E11" s="42" t="s">
+      <c r="E11" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F11" s="42" t="s">
+      <c r="F11" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G11" s="42" t="s">
+      <c r="G11" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H11" t="s">
         <v>98</v>
       </c>
-      <c r="I11" s="43" t="s">
+      <c r="I11" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J11" t="s">
@@ -4615,23 +4596,23 @@
       <c r="O11" t="s">
         <v>102</v>
       </c>
-      <c r="P11" s="44" t="s">
+      <c r="P11" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R11" s="44" t="str">
+      <c r="R11" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S11" s="45" t="s">
+      <c r="S11" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T11" s="44" t="s">
+      <c r="T11" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U11" s="46" t="s">
+      <c r="U11" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V11" s="44" t="e">
+      <c r="V11" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4650,40 +4631,40 @@
       <c r="AA11" t="s">
         <v>109</v>
       </c>
-      <c r="AB11" s="46" t="s">
+      <c r="AB11" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>93</v>
       </c>
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C12" s="27" t="str">
+      <c r="C12" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E12" s="42" t="s">
+      <c r="E12" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F12" s="42" t="s">
+      <c r="F12" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G12" s="42" t="s">
+      <c r="G12" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H12" t="s">
         <v>98</v>
       </c>
-      <c r="I12" s="43" t="s">
+      <c r="I12" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J12" t="s">
@@ -4701,23 +4682,23 @@
       <c r="O12" t="s">
         <v>102</v>
       </c>
-      <c r="P12" s="44" t="s">
+      <c r="P12" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R12" s="44" t="str">
+      <c r="R12" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S12" s="45" t="s">
+      <c r="S12" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T12" s="44" t="s">
+      <c r="T12" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U12" s="46" t="s">
+      <c r="U12" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V12" s="44" t="e">
+      <c r="V12" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4736,40 +4717,40 @@
       <c r="AA12" t="s">
         <v>109</v>
       </c>
-      <c r="AB12" s="46" t="s">
+      <c r="AB12" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:29" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" s="32" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>93</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C13" s="27" t="str">
+      <c r="C13" s="15" t="str">
         <f t="shared" si="0"/>
         <v>&lt;air_date&gt;</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E13" s="42" t="s">
+      <c r="E13" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F13" s="42" t="s">
+      <c r="F13" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G13" s="42" t="s">
+      <c r="G13" s="27" t="s">
         <v>52</v>
       </c>
       <c r="H13" t="s">
         <v>98</v>
       </c>
-      <c r="I13" s="43" t="s">
+      <c r="I13" s="50" t="s">
         <v>99</v>
       </c>
       <c r="J13" t="s">
@@ -4787,23 +4768,23 @@
       <c r="O13" t="s">
         <v>102</v>
       </c>
-      <c r="P13" s="44" t="s">
+      <c r="P13" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="R13" s="44" t="str">
+      <c r="R13" s="51" t="str">
         <f t="shared" si="1"/>
         <v>&lt;gross_rate&gt;</v>
       </c>
-      <c r="S13" s="45" t="s">
+      <c r="S13" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="T13" s="44" t="s">
+      <c r="T13" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="U13" s="46" t="s">
+      <c r="U13" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="V13" s="44" t="e">
+      <c r="V13" s="51" t="e">
         <f t="shared" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -4822,7 +4803,7 @@
       <c r="AA13" t="s">
         <v>109</v>
       </c>
-      <c r="AB13" s="46" t="s">
+      <c r="AB13" s="29" t="s">
         <v>25</v>
       </c>
       <c r="AC13" t="s">
@@ -4830,206 +4811,206 @@
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B14" s="40"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-      <c r="I14" s="43"/>
-      <c r="P14" s="47"/>
-      <c r="R14" s="47"/>
-      <c r="S14" s="45"/>
-      <c r="T14" s="47"/>
-      <c r="U14" s="46"/>
-      <c r="V14" s="47"/>
-      <c r="AB14" s="46"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="I14" s="50"/>
+      <c r="P14" s="52"/>
+      <c r="R14" s="52"/>
+      <c r="S14" s="28"/>
+      <c r="T14" s="52"/>
+      <c r="U14" s="29"/>
+      <c r="V14" s="52"/>
+      <c r="AB14" s="29"/>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B15" s="40"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="I15" s="43"/>
-      <c r="P15" s="47"/>
-      <c r="R15" s="47"/>
-      <c r="S15" s="45"/>
-      <c r="T15" s="47"/>
-      <c r="U15" s="46"/>
-      <c r="V15" s="47"/>
-      <c r="AB15" s="46"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="I15" s="50"/>
+      <c r="P15" s="52"/>
+      <c r="R15" s="52"/>
+      <c r="S15" s="28"/>
+      <c r="T15" s="52"/>
+      <c r="U15" s="29"/>
+      <c r="V15" s="52"/>
+      <c r="AB15" s="29"/>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B16" s="40"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="I16" s="43"/>
-      <c r="P16" s="47"/>
-      <c r="R16" s="47"/>
-      <c r="S16" s="45"/>
-      <c r="T16" s="47"/>
-      <c r="U16" s="46"/>
-      <c r="V16" s="47"/>
-      <c r="AB16" s="46"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="I16" s="50"/>
+      <c r="P16" s="52"/>
+      <c r="R16" s="52"/>
+      <c r="S16" s="28"/>
+      <c r="T16" s="52"/>
+      <c r="U16" s="29"/>
+      <c r="V16" s="52"/>
+      <c r="AB16" s="29"/>
     </row>
     <row r="17" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B17" s="40"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="I17" s="43"/>
-      <c r="P17" s="47"/>
-      <c r="R17" s="47"/>
-      <c r="S17" s="45"/>
-      <c r="T17" s="47"/>
-      <c r="U17" s="46"/>
-      <c r="V17" s="47"/>
-      <c r="AB17" s="46"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="I17" s="50"/>
+      <c r="P17" s="52"/>
+      <c r="R17" s="52"/>
+      <c r="S17" s="28"/>
+      <c r="T17" s="52"/>
+      <c r="U17" s="29"/>
+      <c r="V17" s="52"/>
+      <c r="AB17" s="29"/>
     </row>
     <row r="18" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B18" s="40"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="I18" s="43"/>
-      <c r="P18" s="47"/>
-      <c r="R18" s="47"/>
-      <c r="S18" s="45"/>
-      <c r="T18" s="47"/>
-      <c r="U18" s="46"/>
-      <c r="V18" s="47"/>
-      <c r="AB18" s="46"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="I18" s="50"/>
+      <c r="P18" s="52"/>
+      <c r="R18" s="52"/>
+      <c r="S18" s="28"/>
+      <c r="T18" s="52"/>
+      <c r="U18" s="29"/>
+      <c r="V18" s="52"/>
+      <c r="AB18" s="29"/>
     </row>
     <row r="19" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B19" s="40"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="I19" s="43"/>
-      <c r="P19" s="47"/>
-      <c r="R19" s="47"/>
-      <c r="S19" s="45"/>
-      <c r="T19" s="47"/>
-      <c r="U19" s="46"/>
-      <c r="V19" s="47"/>
-      <c r="AB19" s="46"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="I19" s="50"/>
+      <c r="P19" s="52"/>
+      <c r="R19" s="52"/>
+      <c r="S19" s="28"/>
+      <c r="T19" s="52"/>
+      <c r="U19" s="29"/>
+      <c r="V19" s="52"/>
+      <c r="AB19" s="29"/>
     </row>
     <row r="20" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B20" s="40"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="41"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="I20" s="43"/>
-      <c r="P20" s="47"/>
-      <c r="R20" s="47"/>
-      <c r="S20" s="45"/>
-      <c r="T20" s="47"/>
-      <c r="U20" s="46"/>
-      <c r="V20" s="47"/>
-      <c r="AB20" s="46"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="I20" s="50"/>
+      <c r="P20" s="52"/>
+      <c r="R20" s="52"/>
+      <c r="S20" s="28"/>
+      <c r="T20" s="52"/>
+      <c r="U20" s="29"/>
+      <c r="V20" s="52"/>
+      <c r="AB20" s="29"/>
     </row>
     <row r="21" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B21" s="40"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="I21" s="43"/>
-      <c r="P21" s="47"/>
-      <c r="R21" s="47"/>
-      <c r="S21" s="45"/>
-      <c r="T21" s="47"/>
-      <c r="U21" s="46"/>
-      <c r="V21" s="47"/>
-      <c r="AB21" s="46"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="I21" s="50"/>
+      <c r="P21" s="52"/>
+      <c r="R21" s="52"/>
+      <c r="S21" s="28"/>
+      <c r="T21" s="52"/>
+      <c r="U21" s="29"/>
+      <c r="V21" s="52"/>
+      <c r="AB21" s="29"/>
     </row>
     <row r="22" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B22" s="40"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="41"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="I22" s="43"/>
-      <c r="P22" s="47"/>
-      <c r="R22" s="47"/>
-      <c r="S22" s="45"/>
-      <c r="T22" s="47"/>
-      <c r="U22" s="46"/>
-      <c r="V22" s="47"/>
-      <c r="AB22" s="46"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="I22" s="50"/>
+      <c r="P22" s="52"/>
+      <c r="R22" s="52"/>
+      <c r="S22" s="28"/>
+      <c r="T22" s="52"/>
+      <c r="U22" s="29"/>
+      <c r="V22" s="52"/>
+      <c r="AB22" s="29"/>
     </row>
     <row r="23" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B23" s="40"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="42"/>
-      <c r="I23" s="43"/>
-      <c r="P23" s="47"/>
-      <c r="R23" s="47"/>
-      <c r="S23" s="45"/>
-      <c r="T23" s="47"/>
-      <c r="U23" s="46"/>
-      <c r="V23" s="47"/>
-      <c r="AB23" s="46"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="I23" s="50"/>
+      <c r="P23" s="52"/>
+      <c r="R23" s="52"/>
+      <c r="S23" s="28"/>
+      <c r="T23" s="52"/>
+      <c r="U23" s="29"/>
+      <c r="V23" s="52"/>
+      <c r="AB23" s="29"/>
     </row>
     <row r="24" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B24" s="40"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="42"/>
-      <c r="G24" s="42"/>
-      <c r="I24" s="43"/>
-      <c r="P24" s="47"/>
-      <c r="R24" s="47"/>
-      <c r="S24" s="45"/>
-      <c r="T24" s="47"/>
-      <c r="U24" s="46"/>
-      <c r="V24" s="47"/>
-      <c r="AB24" s="46"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="I24" s="50"/>
+      <c r="P24" s="52"/>
+      <c r="R24" s="52"/>
+      <c r="S24" s="28"/>
+      <c r="T24" s="52"/>
+      <c r="U24" s="29"/>
+      <c r="V24" s="52"/>
+      <c r="AB24" s="29"/>
     </row>
     <row r="25" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B25" s="40"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="41"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="42"/>
-      <c r="G25" s="42"/>
-      <c r="I25" s="43"/>
-      <c r="P25" s="47"/>
-      <c r="R25" s="47"/>
-      <c r="S25" s="45"/>
-      <c r="T25" s="47"/>
-      <c r="U25" s="46"/>
-      <c r="V25" s="47"/>
-      <c r="AB25" s="46"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="I25" s="50"/>
+      <c r="P25" s="52"/>
+      <c r="R25" s="52"/>
+      <c r="S25" s="28"/>
+      <c r="T25" s="52"/>
+      <c r="U25" s="29"/>
+      <c r="V25" s="52"/>
+      <c r="AB25" s="29"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:AC1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5039,7 +5020,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="21" t="s">
         <v>110</v>
       </c>
       <c r="B3" t="s">
@@ -5050,31 +5031,31 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="31" t="s">
         <v>113</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="B5" s="36">
+      <c r="B5" s="22">
         <v>0</v>
       </c>
-      <c r="C5" s="36">
+      <c r="C5" s="22">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="B6" s="36">
+      <c r="B6" s="22">
         <v>0</v>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="22">
         <v>0</v>
       </c>
     </row>

</xml_diff>